<commit_message>
Populate the Cash flow Statement
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-22-tran-vingroup-financials.xlsx
+++ b/models/builds/2026-05-22-tran-vingroup-financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tan\Leanings\VEMBA Hawaii\Corporate_Finance\Corporate-Finance\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22E040D-886B-445E-8473-B2989A6E249A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9221372-EBE9-4329-8823-68DC356C8D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17040" yWindow="3540" windowWidth="24090" windowHeight="27600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22185" yWindow="2610" windowWidth="13860" windowHeight="27600" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="324">
   <si>
     <t>UNIVERSITY OF HAWAIʻI AT MĀNOA · SHIDLER COLLEGE OF BUSINESS</t>
   </si>
@@ -379,9 +379,6 @@
   </si>
   <si>
     <t>Income Statement</t>
-  </si>
-  <si>
-    <t>Current fiscal year · figures in $millions</t>
   </si>
   <si>
     <t>Line Item</t>
@@ -1992,7 +1989,7 @@
     </row>
     <row r="3" spans="2:8" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="47" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2298,23 +2295,23 @@
     </row>
     <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="D5" s="23" t="s">
         <v>86</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" s="19">
         <v>331837561</v>
@@ -2325,7 +2322,7 @@
     </row>
     <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C7" s="19">
         <v>247489507</v>
@@ -2337,7 +2334,7 @@
     </row>
     <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C8" s="19">
         <v>49053914</v>
@@ -2349,7 +2346,7 @@
     </row>
     <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9" s="19">
         <v>31665247</v>
@@ -2361,7 +2358,7 @@
     </row>
     <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C10" s="21">
         <f>C6-C7-C8-C9</f>
@@ -2374,7 +2371,7 @@
     </row>
     <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C11" s="19">
         <v>51968218</v>
@@ -2386,7 +2383,7 @@
     </row>
     <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C12" s="19">
         <v>29159736</v>
@@ -2398,7 +2395,7 @@
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C13" s="21">
         <f>C10+C11-C12</f>
@@ -2411,7 +2408,7 @@
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C14" s="19">
         <v>15372561</v>
@@ -2423,7 +2420,7 @@
     </row>
     <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C15" s="22">
         <f>C13-C14</f>
@@ -2436,12 +2433,12 @@
     </row>
     <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C18" s="19"/>
       <c r="D18" s="25">
@@ -2451,7 +2448,7 @@
     </row>
     <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" s="21">
         <f>C15-C18</f>
@@ -2480,123 +2477,133 @@
   <sheetData>
     <row r="2" spans="2:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>84</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="23" t="s">
-        <v>86</v>
-      </c>
       <c r="D5" s="23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D6" s="15"/>
     </row>
     <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C7" s="27">
         <f>INC_net</f>
         <v>11064814</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" s="27">
         <f>INC_depreciation</f>
         <v>31665247</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="19">
+        <v>-20235943</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>108</v>
-      </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="15" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="C11" s="19"/>
+        <v>109</v>
+      </c>
+      <c r="C11" s="19">
+        <v>-67530856</v>
+      </c>
       <c r="D11" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="C12" s="19"/>
+        <v>110</v>
+      </c>
+      <c r="C12" s="19">
+        <v>3985858</v>
+      </c>
       <c r="D12" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C13" s="19"/>
+        <v>111</v>
+      </c>
+      <c r="C13" s="19">
+        <v>12750861</v>
+      </c>
       <c r="D13" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C14" s="19"/>
+        <v>112</v>
+      </c>
+      <c r="C14" s="19">
+        <v>97154801</v>
+      </c>
       <c r="D14" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C15" s="21">
         <f>SUM(C10:C14)</f>
-        <v>0</v>
+        <v>26124721</v>
       </c>
       <c r="D15" s="15"/>
     </row>
     <row r="16" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C16" s="22">
         <f>C7+C8+C15</f>
-        <v>42730061</v>
+        <v>68854782</v>
       </c>
       <c r="D16" s="15"/>
     </row>
@@ -2605,38 +2612,44 @@
     </row>
     <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D18" s="15"/>
     </row>
     <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="C19" s="19"/>
+        <v>116</v>
+      </c>
+      <c r="C19" s="19">
+        <v>-76157072</v>
+      </c>
       <c r="D19" s="15"/>
     </row>
     <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="19"/>
+        <v>117</v>
+      </c>
+      <c r="C20" s="19">
+        <v>65772180</v>
+      </c>
       <c r="D20" s="15"/>
     </row>
     <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="C21" s="19"/>
+        <v>118</v>
+      </c>
+      <c r="C21" s="19">
+        <v>-129543511</v>
+      </c>
       <c r="D21" s="15"/>
     </row>
     <row r="22" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C22" s="22">
         <f>SUM(C19:C21)</f>
-        <v>0</v>
+        <v>-139928403</v>
       </c>
       <c r="D22" s="15"/>
     </row>
@@ -2645,52 +2658,63 @@
     </row>
     <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D24" s="15"/>
     </row>
     <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C25" s="19"/>
+        <v>121</v>
+      </c>
+      <c r="C25" s="19">
+        <v>18811339</v>
+      </c>
       <c r="D25" s="15"/>
     </row>
     <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C26" s="19"/>
+        <v>122</v>
+      </c>
+      <c r="C26" s="19">
+        <v>83383279</v>
+      </c>
       <c r="D26" s="15"/>
     </row>
     <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27" s="19"/>
+        <v>123</v>
+      </c>
+      <c r="C27" s="19">
+        <v>-2577141</v>
+      </c>
       <c r="D27" s="15"/>
     </row>
     <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="C28" s="19"/>
+        <v>124</v>
+      </c>
+      <c r="C28" s="19">
+        <v>2267028</v>
+      </c>
       <c r="D28" s="15"/>
     </row>
     <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="C29" s="19"/>
+        <v>125</v>
+      </c>
+      <c r="C29" s="19">
+        <f>-265382+390107</f>
+        <v>124725</v>
+      </c>
       <c r="D29" s="15"/>
     </row>
     <row r="30" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C30" s="22">
         <f>SUM(C25:C29)</f>
-        <v>0</v>
+        <v>102009230</v>
       </c>
       <c r="D30" s="15"/>
     </row>
@@ -2699,11 +2723,11 @@
     </row>
     <row r="32" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C32" s="22">
         <f>C16+C22+C30</f>
-        <v>42730061</v>
+        <v>30935609</v>
       </c>
       <c r="D32" s="15"/>
     </row>
@@ -2727,117 +2751,117 @@
   <sheetData>
     <row r="2" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="D5" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="E5" s="23" t="s">
         <v>133</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C6" s="29">
         <v>2024</v>
       </c>
       <c r="D6" s="30"/>
       <c r="E6" s="30" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C7" s="31">
         <f>yearCurrent-1</f>
         <v>2023</v>
       </c>
       <c r="D7" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="E7" s="30" t="s">
         <v>138</v>
-      </c>
-      <c r="E7" s="30" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C8" s="32"/>
       <c r="D8" s="30"/>
       <c r="E8" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C9" s="33"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C10" s="34">
         <v>0.09</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C11" s="34">
         <v>0.21</v>
       </c>
       <c r="D11" s="30"/>
       <c r="E11" s="30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C12" s="35">
         <f>share_price*shares_outstanding</f>
         <v>0</v>
       </c>
       <c r="D12" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="E12" s="30" t="s">
         <v>149</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="54" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C14" s="49"/>
       <c r="D14" s="49"/>
@@ -2845,82 +2869,82 @@
     </row>
     <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C15" s="36">
         <f>BAL_equity_shareholders_prior</f>
         <v>153834481</v>
       </c>
       <c r="D15" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="E15" s="30" t="s">
         <v>153</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C16" s="36">
         <f>BAL_inventories_prior</f>
         <v>114090183</v>
       </c>
       <c r="D16" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="E16" s="30" t="s">
         <v>156</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C17" s="36">
         <f>BAL_receivables_prior</f>
         <v>190046565</v>
       </c>
       <c r="D17" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="E17" s="30" t="s">
         <v>159</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C18" s="36">
         <f>BAL_assets_total_prior</f>
         <v>836603903</v>
       </c>
       <c r="D18" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="E18" s="30" t="s">
         <v>162</v>
-      </c>
-      <c r="E18" s="30" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C19" s="36">
         <f>BAL_debt_long_term_prior+BAL_equity_shareholders_prior</f>
         <v>286565393</v>
       </c>
       <c r="D19" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="E19" s="30" t="s">
         <v>165</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="54" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C21" s="49"/>
       <c r="D21" s="49"/>
@@ -2928,107 +2952,107 @@
     </row>
     <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C22" s="36">
         <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
         <v>34101005.439999998</v>
       </c>
       <c r="D22" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="E22" s="30" t="s">
         <v>169</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C23" s="37">
         <f>IFERROR(INC_sales/365,"")</f>
         <v>909144.00273972598</v>
       </c>
       <c r="D23" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="E23" s="30" t="s">
         <v>172</v>
-      </c>
-      <c r="E23" s="30" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C24" s="36">
         <f>BAL_equity_shareholders_curr</f>
         <v>151488935</v>
       </c>
       <c r="D24" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="30" t="s">
         <v>175</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="12" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C25" s="36">
         <f>BAL_cash_marketable_securities_curr</f>
         <v>83380686</v>
       </c>
       <c r="D25" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="E25" s="30" t="s">
         <v>178</v>
-      </c>
-      <c r="E25" s="30" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C26" s="36">
         <f>BAL_assets_current_curr</f>
         <v>658772464</v>
       </c>
       <c r="D26" s="30" t="s">
+        <v>180</v>
+      </c>
+      <c r="E26" s="30" t="s">
         <v>181</v>
-      </c>
-      <c r="E26" s="30" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C27" s="36">
         <f>BAL_liabilities_current_curr</f>
         <v>587454564</v>
       </c>
       <c r="D27" s="30" t="s">
+        <v>183</v>
+      </c>
+      <c r="E27" s="30" t="s">
         <v>184</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C28" s="37">
         <f>IFERROR(INC_cost_goods_sold/365,"")</f>
         <v>678053.44383561646</v>
       </c>
       <c r="D28" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="E28" s="30" t="s">
         <v>187</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3040,75 +3064,75 @@
         <v>224500548</v>
       </c>
       <c r="D29" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="E29" s="30" t="s">
         <v>189</v>
-      </c>
-      <c r="E29" s="30" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="12" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C30" s="36">
         <f>BAL_assets_current_curr-BAL_liabilities_current_curr</f>
         <v>71317900</v>
       </c>
       <c r="D30" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="E30" s="30" t="s">
         <v>192</v>
-      </c>
-      <c r="E30" s="30" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C31" s="36">
         <f>BAL_assets_total_curr</f>
         <v>1118622625</v>
       </c>
       <c r="D31" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="E31" s="30" t="s">
         <v>195</v>
-      </c>
-      <c r="E31" s="30" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C32" s="36">
         <f>BAL_debt_long_term_curr+BAL_equity_shareholders_curr</f>
         <v>375989483</v>
       </c>
       <c r="D32" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="E32" s="30" t="s">
         <v>198</v>
-      </c>
-      <c r="E32" s="30" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C33" s="36">
         <f>BAL_liabilities_total_curr</f>
         <v>967133690</v>
       </c>
       <c r="D33" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="E33" s="30" t="s">
         <v>201</v>
-      </c>
-      <c r="E33" s="30" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="54" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C35" s="49"/>
       <c r="D35" s="49"/>
@@ -3116,69 +3140,69 @@
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C36" s="37">
         <f>AVERAGE(startYear_equity,currentYear_equity)</f>
         <v>152661708</v>
       </c>
       <c r="D36" s="30" t="s">
+        <v>204</v>
+      </c>
+      <c r="E36" s="30" t="s">
         <v>205</v>
-      </c>
-      <c r="E36" s="30" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C37" s="37">
         <f>AVERAGE(startYear_total_assets,currentYear_assets_total)</f>
         <v>977613264</v>
       </c>
       <c r="D37" s="30" t="s">
+        <v>207</v>
+      </c>
+      <c r="E37" s="30" t="s">
         <v>208</v>
-      </c>
-      <c r="E37" s="30" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C38" s="37">
         <f>AVERAGE(startYear_total_capitalization,currentYear_total_capitalization)</f>
         <v>331277438</v>
       </c>
       <c r="D38" s="30" t="s">
+        <v>210</v>
+      </c>
+      <c r="E38" s="30" t="s">
         <v>211</v>
-      </c>
-      <c r="E38" s="30" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="C41" s="23" t="s">
         <v>213</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="D41" s="23" t="s">
         <v>214</v>
       </c>
-      <c r="D41" s="23" t="s">
+      <c r="E41" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="F41" s="23" t="s">
         <v>215</v>
-      </c>
-      <c r="E41" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="F41" s="23" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -3186,37 +3210,37 @@
     </row>
     <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="12" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C43" s="38"/>
       <c r="D43" s="30" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E43" s="30"/>
     </row>
     <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C44" s="39"/>
       <c r="D44" s="30" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E44" s="30"/>
     </row>
     <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C45" s="38"/>
       <c r="D45" s="30" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E45" s="30"/>
     </row>
     <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -3224,67 +3248,67 @@
     </row>
     <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C47" s="40"/>
       <c r="D47" s="30" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E47" s="30"/>
     </row>
     <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="12" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C48" s="40"/>
       <c r="D48" s="30" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E48" s="30"/>
     </row>
     <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C49" s="40"/>
       <c r="D49" s="30" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E49" s="30"/>
     </row>
     <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C50" s="40"/>
       <c r="D50" s="30" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E50" s="30"/>
     </row>
     <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C51" s="40"/>
       <c r="D51" s="30" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E51" s="30"/>
     </row>
     <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="12" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C52" s="40"/>
       <c r="D52" s="30" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E52" s="30"/>
     </row>
     <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -3292,81 +3316,81 @@
     </row>
     <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="12" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C54" s="39"/>
       <c r="D54" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="E54" s="30" t="s">
         <v>239</v>
-      </c>
-      <c r="E54" s="30" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C55" s="39"/>
       <c r="D55" s="30" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E55" s="30"/>
     </row>
     <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="12" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C56" s="41"/>
       <c r="D56" s="30" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E56" s="30"/>
     </row>
     <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C57" s="39"/>
       <c r="D57" s="30" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E57" s="30"/>
     </row>
     <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C58" s="41"/>
       <c r="D58" s="30" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E58" s="30"/>
     </row>
     <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="12" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C59" s="40"/>
       <c r="D59" s="30" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E59" s="30"/>
     </row>
     <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C60" s="40"/>
       <c r="D60" s="30" t="s">
+        <v>251</v>
+      </c>
+      <c r="E60" s="30" t="s">
         <v>252</v>
-      </c>
-      <c r="E60" s="30" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -3374,81 +3398,81 @@
     </row>
     <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C62" s="40"/>
       <c r="D62" s="30" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E62" s="30"/>
     </row>
     <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C63" s="39"/>
       <c r="D63" s="30" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E63" s="30"/>
     </row>
     <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C64" s="40"/>
       <c r="D64" s="30" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E64" s="30"/>
     </row>
     <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C65" s="39"/>
       <c r="D65" s="30" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E65" s="30"/>
     </row>
     <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="12" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C66" s="39"/>
       <c r="D66" s="30" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E66" s="30"/>
     </row>
     <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C67" s="42"/>
       <c r="D67" s="30" t="s">
+        <v>265</v>
+      </c>
+      <c r="E67" s="30" t="s">
         <v>266</v>
-      </c>
-      <c r="E67" s="30" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C68" s="39"/>
       <c r="D68" s="30" t="s">
+        <v>268</v>
+      </c>
+      <c r="E68" s="30" t="s">
         <v>269</v>
-      </c>
-      <c r="E68" s="30" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -3456,47 +3480,47 @@
     </row>
     <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C70" s="40"/>
       <c r="D70" s="30" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E70" s="30"/>
     </row>
     <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C71" s="39"/>
       <c r="D71" s="30" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E71" s="30"/>
     </row>
     <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C72" s="39"/>
       <c r="D72" s="30" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E72" s="30"/>
     </row>
     <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C73" s="39"/>
       <c r="D73" s="30" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E73" s="30"/>
     </row>
     <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -3504,11 +3528,11 @@
     </row>
     <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C75" s="40"/>
       <c r="D75" s="30" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E75" s="30"/>
       <c r="F75" s="44" t="str">
@@ -3518,11 +3542,11 @@
     </row>
     <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C76" s="40"/>
       <c r="D76" s="30" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E76" s="30"/>
     </row>
@@ -3548,156 +3572,156 @@
   <sheetData>
     <row r="2" spans="2:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
+        <v>285</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>286</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="43" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>288</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="43" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="43" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="43" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="45" x14ac:dyDescent="0.25">
       <c r="B9" s="43" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="43" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B11" s="43" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="90" x14ac:dyDescent="0.25">
       <c r="B12" s="43" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="43" t="s">
+        <v>296</v>
+      </c>
+      <c r="C13" s="45" t="s">
         <v>297</v>
-      </c>
-      <c r="C13" s="45" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="45" x14ac:dyDescent="0.25">
       <c r="B14" s="43" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="43" t="s">
+        <v>299</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>300</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="43" t="s">
+        <v>301</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>302</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="43" t="s">
+        <v>303</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>304</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="43" t="s">
+        <v>305</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>306</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="43" t="s">
+        <v>307</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>308</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="43" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="43" t="s">
+        <v>310</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>311</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="43" t="s">
+        <v>312</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>313</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Populate the Income Statement and Cash Flow Statement for FY Prior missed
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-22-tran-vingroup-financials.xlsx
+++ b/models/builds/2026-05-22-tran-vingroup-financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tan\Leanings\VEMBA Hawaii\Corporate_Finance\Corporate-Finance\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9221372-EBE9-4329-8823-68DC356C8D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03B8724E-10E3-4F69-A915-D11F597DE356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22185" yWindow="2610" windowWidth="13860" windowHeight="27600" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22185" yWindow="2610" windowWidth="13860" windowHeight="27600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="324">
   <si>
     <t>UNIVERSITY OF HAWAIʻI AT MĀNOA · SHIDLER COLLEGE OF BUSINESS</t>
   </si>
@@ -382,12 +382,6 @@
   </si>
   <si>
     <t>Line Item</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
-    <t>% of Sales</t>
   </si>
   <si>
     <t>Net sales</t>
@@ -1104,6 +1098,14 @@
   </si>
   <si>
     <t>Current fiscal year · figures in VND millions</t>
+  </si>
+  <si>
+    <t>% of Sales
+in FY Current</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of Sales
+in FY Prior </t>
   </si>
 </sst>
 </file>
@@ -1317,7 +1319,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1411,6 +1413,18 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1989,7 +2003,7 @@
     </row>
     <row r="3" spans="2:8" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="47" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2279,184 +2293,278 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B2:D19"/>
+  <dimension ref="B2:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="3" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" s="58" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="56" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="57" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="57" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="55" t="s">
+        <v>322</v>
+      </c>
+      <c r="F5" s="55" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="23" t="s">
+    <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="12" t="s">
         <v>85</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="12" t="s">
-        <v>87</v>
       </c>
       <c r="C6" s="19">
         <v>331837561</v>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="19">
+        <v>189068040</v>
+      </c>
+      <c r="E6" s="24">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F6" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C7" s="19">
         <v>247489507</v>
       </c>
-      <c r="D7" s="25">
-        <f t="shared" ref="D7:D15" si="0">IFERROR(C7/$C$6,"")</f>
+      <c r="D7" s="19">
+        <v>139140098</v>
+      </c>
+      <c r="E7" s="25">
+        <f>IFERROR(C7/$C$6,"")</f>
         <v>0.74581523036206265</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F7" s="25">
+        <f>IFERROR(D7/$D$6,"")</f>
+        <v>0.73592606132691707</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C8" s="19">
         <v>49053914</v>
       </c>
-      <c r="D8" s="25">
-        <f t="shared" si="0"/>
+      <c r="D8" s="19">
+        <v>33202226</v>
+      </c>
+      <c r="E8" s="25">
+        <f>IFERROR(C8/$C$6,"")</f>
         <v>0.1478250799944856</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F8" s="25">
+        <f t="shared" ref="F8:F14" si="0">IFERROR(D8/$D$6,"")</f>
+        <v>0.17560993386296278</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C9" s="19">
         <v>31665247</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="19">
+        <v>22627124</v>
+      </c>
+      <c r="E9" s="25">
+        <f>IFERROR(C9/$C$6,"")</f>
+        <v>9.5423938461264179E-2</v>
+      </c>
+      <c r="F9" s="25">
         <f t="shared" si="0"/>
-        <v>9.5423938461264179E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0.1196771490305818</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C10" s="21">
         <f>C6-C7-C8-C9</f>
         <v>3628893</v>
       </c>
-      <c r="D10" s="25">
+      <c r="D10" s="21">
+        <f>D6-D7-D8-D9</f>
+        <v>-5901408</v>
+      </c>
+      <c r="E10" s="25">
+        <f>IFERROR(C10/$C$6,"")</f>
+        <v>1.0935751182187601E-2</v>
+      </c>
+      <c r="F10" s="25">
         <f t="shared" si="0"/>
-        <v>1.0935751182187601E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>-3.1213144220461585E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C11" s="19">
         <v>51968218</v>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="19">
+        <v>45620158</v>
+      </c>
+      <c r="E11" s="25">
+        <f>IFERROR(C11/$C$6,"")</f>
+        <v>0.15660740105307128</v>
+      </c>
+      <c r="F11" s="25">
         <f t="shared" si="0"/>
-        <v>0.15660740105307128</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0.24128963308658619</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C12" s="19">
         <v>29159736</v>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="19">
+        <v>22980044</v>
+      </c>
+      <c r="E12" s="25">
+        <f>IFERROR(C12/$C$6,"")</f>
+        <v>8.7873524359709243E-2</v>
+      </c>
+      <c r="F12" s="25">
         <f t="shared" si="0"/>
-        <v>8.7873524359709243E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0.12154377863122715</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="20" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C13" s="21">
         <f>C10+C11-C12</f>
         <v>26437375</v>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="21">
+        <f>D10+D11-D12</f>
+        <v>16738706</v>
+      </c>
+      <c r="E13" s="25">
+        <f>IFERROR(C13/$C$6,"")</f>
+        <v>7.9669627875549626E-2</v>
+      </c>
+      <c r="F13" s="25">
         <f t="shared" si="0"/>
-        <v>7.9669627875549626E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>8.8532710234897449E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C14" s="19">
         <v>15372561</v>
       </c>
-      <c r="D14" s="25">
+      <c r="D14" s="19">
+        <v>11462648</v>
+      </c>
+      <c r="E14" s="25">
+        <f>IFERROR(C14/$C$6,"")</f>
+        <v>4.6325560475054241E-2</v>
+      </c>
+      <c r="F14" s="25">
         <f t="shared" si="0"/>
-        <v>4.6325560475054241E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>6.0627105458965991E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C15" s="22">
         <f>C13-C14</f>
         <v>11064814</v>
       </c>
-      <c r="D15" s="26">
-        <f t="shared" si="0"/>
+      <c r="D15" s="22">
+        <f>D13-D14</f>
+        <v>5276058</v>
+      </c>
+      <c r="E15" s="26">
+        <f>IFERROR(C15/$C$6,"")</f>
         <v>3.3344067400495392E-2</v>
       </c>
-    </row>
-    <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F15" s="26">
+        <f>IFERROR(D15/$D$6,"")</f>
+        <v>2.7905604775931458E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="18" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C18" s="19"/>
-      <c r="D18" s="25">
+      <c r="D18" s="19">
+        <v>666188</v>
+      </c>
+      <c r="E18" s="25">
         <f>IFERROR(C18/$C$6,"")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="25">
+        <f>IFERROR(D18/$D$6,"")</f>
+        <v>3.5235357599306578E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="20" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C19" s="21">
         <f>C15-C18</f>
         <v>11064814</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="21">
+        <f>D15-D18</f>
+        <v>4609870</v>
+      </c>
+      <c r="E19" s="25">
         <f>IFERROR(C19/$C$6,"")</f>
         <v>3.3344067400495392E-2</v>
+      </c>
+      <c r="F19" s="25">
+        <f>IFERROR(D19/$D$6,"")</f>
+        <v>2.4382069016000801E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2466,270 +2574,338 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B2:D32"/>
+  <dimension ref="B2:E32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="3" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D5" s="23" t="s">
+      <c r="C5" s="57" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="57" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="E6" s="15"/>
+    </row>
+    <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="12" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="D6" s="15"/>
-    </row>
-    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="12" t="s">
-        <v>103</v>
       </c>
       <c r="C7" s="27">
         <f>INC_net</f>
         <v>11064814</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="27">
+        <v>5276058</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C8" s="27">
         <f>INC_depreciation</f>
         <v>31665247</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="27">
+        <v>22627124</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="28" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" s="15"/>
-    </row>
-    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E9" s="15"/>
+    </row>
+    <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C10" s="19">
         <v>-20235943</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="19">
+        <v>-95017737</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C11" s="19">
         <v>-67530856</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="19">
+        <v>-23011001</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="12" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="12" t="s">
-        <v>110</v>
       </c>
       <c r="C12" s="19">
         <v>3985858</v>
       </c>
-      <c r="D12" s="15" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D12" s="19">
+        <v>-3116968</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C13" s="19">
         <v>12750861</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D13" s="19">
+        <v>10160792</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C14" s="19">
         <v>97154801</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D14" s="19">
+        <v>99548789</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="20" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C15" s="21">
         <f>SUM(C10:C14)</f>
         <v>26124721</v>
       </c>
-      <c r="D15" s="15"/>
-    </row>
-    <row r="16" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D15" s="21">
+        <f>SUM(D10:D14)</f>
+        <v>-11436125</v>
+      </c>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C16" s="22">
         <f>C7+C8+C15</f>
         <v>68854782</v>
       </c>
-      <c r="D16" s="15"/>
-    </row>
-    <row r="17" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D17" s="15"/>
-    </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D16" s="22">
+        <f>D7+D8+D15</f>
+        <v>16467057</v>
+      </c>
+      <c r="E16" s="15"/>
+    </row>
+    <row r="17" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="D18" s="15"/>
-    </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+      <c r="E18" s="15"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C19" s="19">
         <v>-76157072</v>
       </c>
-      <c r="D19" s="15"/>
-    </row>
-    <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D19" s="19">
+        <v>-48567437</v>
+      </c>
+      <c r="E19" s="15"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C20" s="19">
         <v>65772180</v>
       </c>
-      <c r="D20" s="15"/>
-    </row>
-    <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D20" s="19">
+        <v>84186330</v>
+      </c>
+      <c r="E20" s="15"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C21" s="19">
         <v>-129543511</v>
       </c>
-      <c r="D21" s="15"/>
-    </row>
-    <row r="22" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="19">
+        <v>-52461980</v>
+      </c>
+      <c r="E21" s="15"/>
+    </row>
+    <row r="22" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C22" s="22">
         <f>SUM(C19:C21)</f>
         <v>-139928403</v>
       </c>
-      <c r="D22" s="15"/>
-    </row>
-    <row r="23" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D23" s="15"/>
-    </row>
-    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D22" s="22">
+        <f>SUM(D19:D21)</f>
+        <v>-16843087</v>
+      </c>
+      <c r="E22" s="15"/>
+    </row>
+    <row r="23" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="E23" s="15"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="D24" s="15"/>
-    </row>
-    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+      <c r="E24" s="15"/>
+    </row>
+    <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C25" s="19">
         <v>18811339</v>
       </c>
-      <c r="D25" s="15"/>
-    </row>
-    <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D25" s="19">
+        <v>-21046056</v>
+      </c>
+      <c r="E25" s="15"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C26" s="19">
         <v>83383279</v>
       </c>
-      <c r="D26" s="15"/>
-    </row>
-    <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D26" s="19">
+        <v>27601580</v>
+      </c>
+      <c r="E26" s="15"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C27" s="19">
         <v>-2577141</v>
       </c>
-      <c r="D27" s="15"/>
-    </row>
-    <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D27" s="19">
+        <v>-666188</v>
+      </c>
+      <c r="E27" s="15"/>
+    </row>
+    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C28" s="19">
         <v>2267028</v>
       </c>
-      <c r="D28" s="15"/>
-    </row>
-    <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D28" s="19">
+        <v>15659006</v>
+      </c>
+      <c r="E28" s="15"/>
+    </row>
+    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C29" s="19">
         <f>-265382+390107</f>
         <v>124725</v>
       </c>
-      <c r="D29" s="15"/>
-    </row>
-    <row r="30" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D29" s="19">
+        <v>-6234548</v>
+      </c>
+      <c r="E29" s="15"/>
+    </row>
+    <row r="30" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C30" s="22">
         <f>SUM(C25:C29)</f>
         <v>102009230</v>
       </c>
-      <c r="D30" s="15"/>
-    </row>
-    <row r="31" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="D31" s="15"/>
-    </row>
-    <row r="32" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D30" s="22">
+        <f>SUM(D25:D29)</f>
+        <v>15313794</v>
+      </c>
+      <c r="E30" s="15"/>
+    </row>
+    <row r="31" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="E31" s="15"/>
+    </row>
+    <row r="32" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C32" s="22">
         <f>C16+C22+C30</f>
         <v>30935609</v>
       </c>
-      <c r="D32" s="15"/>
+      <c r="D32" s="22">
+        <f>D16+D22+D30</f>
+        <v>14937764</v>
+      </c>
+      <c r="E32" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2751,117 +2927,117 @@
   <sheetData>
     <row r="2" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="E5" s="23" t="s">
         <v>131</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C6" s="29">
         <v>2024</v>
       </c>
       <c r="D6" s="30"/>
       <c r="E6" s="30" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C7" s="31">
         <f>yearCurrent-1</f>
         <v>2023</v>
       </c>
       <c r="D7" s="30" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C8" s="32"/>
       <c r="D8" s="30"/>
       <c r="E8" s="30" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C9" s="33"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C10" s="34">
         <v>0.09</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="30" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C11" s="34">
         <v>0.21</v>
       </c>
       <c r="D11" s="30"/>
       <c r="E11" s="30" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C12" s="35">
         <f>share_price*shares_outstanding</f>
         <v>0</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="54" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C14" s="49"/>
       <c r="D14" s="49"/>
@@ -2869,82 +3045,82 @@
     </row>
     <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C15" s="36">
         <f>BAL_equity_shareholders_prior</f>
         <v>153834481</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E15" s="30" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C16" s="36">
         <f>BAL_inventories_prior</f>
         <v>114090183</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C17" s="36">
         <f>BAL_receivables_prior</f>
         <v>190046565</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C18" s="36">
         <f>BAL_assets_total_prior</f>
         <v>836603903</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C19" s="36">
         <f>BAL_debt_long_term_prior+BAL_equity_shareholders_prior</f>
         <v>286565393</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="54" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C21" s="49"/>
       <c r="D21" s="49"/>
@@ -2952,107 +3128,107 @@
     </row>
     <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C22" s="36">
         <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
         <v>34101005.439999998</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="12" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C23" s="37">
         <f>IFERROR(INC_sales/365,"")</f>
         <v>909144.00273972598</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E23" s="30" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="12" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C24" s="36">
         <f>BAL_equity_shareholders_curr</f>
         <v>151488935</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C25" s="36">
         <f>BAL_cash_marketable_securities_curr</f>
         <v>83380686</v>
       </c>
       <c r="D25" s="30" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E25" s="30" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C26" s="36">
         <f>BAL_assets_current_curr</f>
         <v>658772464</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E26" s="30" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C27" s="36">
         <f>BAL_liabilities_current_curr</f>
         <v>587454564</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C28" s="37">
         <f>IFERROR(INC_cost_goods_sold/365,"")</f>
         <v>678053.44383561646</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3064,75 +3240,75 @@
         <v>224500548</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C30" s="36">
         <f>BAL_assets_current_curr-BAL_liabilities_current_curr</f>
         <v>71317900</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E30" s="30" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C31" s="36">
         <f>BAL_assets_total_curr</f>
         <v>1118622625</v>
       </c>
       <c r="D31" s="30" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E31" s="30" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="12" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C32" s="36">
         <f>BAL_debt_long_term_curr+BAL_equity_shareholders_curr</f>
         <v>375989483</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E32" s="30" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="12" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C33" s="36">
         <f>BAL_liabilities_total_curr</f>
         <v>967133690</v>
       </c>
       <c r="D33" s="30" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E33" s="30" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="54" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C35" s="49"/>
       <c r="D35" s="49"/>
@@ -3140,69 +3316,69 @@
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C36" s="37">
         <f>AVERAGE(startYear_equity,currentYear_equity)</f>
         <v>152661708</v>
       </c>
       <c r="D36" s="30" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E36" s="30" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C37" s="37">
         <f>AVERAGE(startYear_total_assets,currentYear_assets_total)</f>
         <v>977613264</v>
       </c>
       <c r="D37" s="30" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E37" s="30" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C38" s="37">
         <f>AVERAGE(startYear_total_capitalization,currentYear_total_capitalization)</f>
         <v>331277438</v>
       </c>
       <c r="D38" s="30" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E38" s="30" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="C41" s="23" t="s">
+        <v>211</v>
+      </c>
+      <c r="D41" s="23" t="s">
         <v>212</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="E41" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="F41" s="23" t="s">
         <v>213</v>
-      </c>
-      <c r="D41" s="23" t="s">
-        <v>214</v>
-      </c>
-      <c r="E41" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="F41" s="23" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -3210,37 +3386,37 @@
     </row>
     <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="12" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C43" s="38"/>
       <c r="D43" s="30" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E43" s="30"/>
     </row>
     <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="12" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C44" s="39"/>
       <c r="D44" s="30" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E44" s="30"/>
     </row>
     <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="12" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C45" s="38"/>
       <c r="D45" s="30" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E45" s="30"/>
     </row>
     <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -3248,67 +3424,67 @@
     </row>
     <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="12" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C47" s="40"/>
       <c r="D47" s="30" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E47" s="30"/>
     </row>
     <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="12" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C48" s="40"/>
       <c r="D48" s="30" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E48" s="30"/>
     </row>
     <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="12" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C49" s="40"/>
       <c r="D49" s="30" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E49" s="30"/>
     </row>
     <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C50" s="40"/>
       <c r="D50" s="30" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E50" s="30"/>
     </row>
     <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="12" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C51" s="40"/>
       <c r="D51" s="30" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E51" s="30"/>
     </row>
     <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="12" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C52" s="40"/>
       <c r="D52" s="30" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E52" s="30"/>
     </row>
     <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -3316,81 +3492,81 @@
     </row>
     <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="12" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C54" s="39"/>
       <c r="D54" s="30" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E54" s="30" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="12" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C55" s="39"/>
       <c r="D55" s="30" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E55" s="30"/>
     </row>
     <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C56" s="41"/>
       <c r="D56" s="30" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E56" s="30"/>
     </row>
     <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="12" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C57" s="39"/>
       <c r="D57" s="30" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E57" s="30"/>
     </row>
     <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="12" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C58" s="41"/>
       <c r="D58" s="30" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E58" s="30"/>
     </row>
     <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="12" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C59" s="40"/>
       <c r="D59" s="30" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E59" s="30"/>
     </row>
     <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="12" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C60" s="40"/>
       <c r="D60" s="30" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E60" s="30" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -3398,81 +3574,81 @@
     </row>
     <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="12" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C62" s="40"/>
       <c r="D62" s="30" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E62" s="30"/>
     </row>
     <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="12" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C63" s="39"/>
       <c r="D63" s="30" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E63" s="30"/>
     </row>
     <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="12" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C64" s="40"/>
       <c r="D64" s="30" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E64" s="30"/>
     </row>
     <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="12" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C65" s="39"/>
       <c r="D65" s="30" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E65" s="30"/>
     </row>
     <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="12" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C66" s="39"/>
       <c r="D66" s="30" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E66" s="30"/>
     </row>
     <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="12" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C67" s="42"/>
       <c r="D67" s="30" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E67" s="30" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="12" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C68" s="39"/>
       <c r="D68" s="30" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E68" s="30" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -3480,47 +3656,47 @@
     </row>
     <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C70" s="40"/>
       <c r="D70" s="30" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E70" s="30"/>
     </row>
     <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="12" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C71" s="39"/>
       <c r="D71" s="30" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E71" s="30"/>
     </row>
     <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C72" s="39"/>
       <c r="D72" s="30" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E72" s="30"/>
     </row>
     <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="12" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C73" s="39"/>
       <c r="D73" s="30" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E73" s="30"/>
     </row>
     <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -3528,11 +3704,11 @@
     </row>
     <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="12" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C75" s="40"/>
       <c r="D75" s="30" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E75" s="30"/>
       <c r="F75" s="44" t="str">
@@ -3542,11 +3718,11 @@
     </row>
     <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="12" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C76" s="40"/>
       <c r="D76" s="30" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E76" s="30"/>
     </row>
@@ -3572,156 +3748,156 @@
   <sheetData>
     <row r="2" spans="2:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="43" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="43" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C6" s="45" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="43" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C7" s="45" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="43" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C8" s="45" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="45" x14ac:dyDescent="0.25">
       <c r="B9" s="43" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="43" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C10" s="45" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B11" s="43" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="90" x14ac:dyDescent="0.25">
       <c r="B12" s="43" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="43" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C13" s="45" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="45" x14ac:dyDescent="0.25">
       <c r="B14" s="43" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C14" s="45" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="43" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="43" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="43" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="43" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="43" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="43" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="43" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="43" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update the Ratios tab
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-22-tran-vingroup-financials.xlsx
+++ b/models/builds/2026-05-22-tran-vingroup-financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tan\Leanings\VEMBA Hawaii\Corporate_Finance\Corporate-Finance\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7190153-C2D0-4874-8A12-FD97A1BE94DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AEC2B0E-D590-48BD-866D-C2296869B154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22185" yWindow="2610" windowWidth="13860" windowHeight="27600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22185" yWindow="2610" windowWidth="13860" windowHeight="27600" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -540,9 +540,6 @@
     <t>yearStart</t>
   </si>
   <si>
-    <t>Share price</t>
-  </si>
-  <si>
     <t>share_price</t>
   </si>
   <si>
@@ -562,9 +559,6 @@
   </si>
   <si>
     <t>tax_rate</t>
-  </si>
-  <si>
-    <t>Market capitalization</t>
   </si>
   <si>
     <t>share_price × shares_outstanding</t>
@@ -1073,9 +1067,6 @@
 - Cost of debt of 9-10% (Vingroup coupon rates)</t>
   </si>
   <si>
-    <t>7,706.031 million shares (7,706,031,024 shares), total shares outstanding as of FY2025. Source: Vingroup FY2025 Annual Report. Implied market cap: VND 1,308,182 billion (~USD 51.4 billion at 25,450 VND/USD).</t>
-  </si>
-  <si>
     <t>Vingroup Annual Report 2025 (audited consolidated financials, VAS) — https://vingroup.net/en/investor-relations | HOSE disclosure portal | VinFast Nasdaq disclosures: investors.vinfastauto.com</t>
   </si>
   <si>
@@ -1139,23 +1130,33 @@
   </si>
   <si>
     <t>31 December 2025 (FY Current) / 31 December 2024 (FY Prior)</t>
+  </si>
+  <si>
+    <t>Share price (VND/share)</t>
+  </si>
+  <si>
+    <t>7,706 million shares (7,706,031,024 shares), total shares outstanding as of FY2025. Source: Vingroup FY2025 Annual Report. Implied market cap: VND 1,308,182 billion (~USD 51.4 billion at 25,450 VND/USD).</t>
+  </si>
+  <si>
+    <t>Market capitalization (VND million)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="9">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;—&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);&quot;—&quot;"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.00;\(#,##0.00\);&quot;—&quot;"/>
     <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="170" formatCode="0.0&quot; days&quot;"/>
     <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="177" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1281,6 +1282,13 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1354,8 +1362,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1410,7 +1419,6 @@
     <xf numFmtId="1" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1463,12 +1471,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="8" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1783,32 +1793,32 @@
       <c r="C2" s="1"/>
     </row>
     <row r="4" spans="2:3" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="49"/>
+      <c r="C4" s="48"/>
     </row>
     <row r="5" spans="2:3" ht="26.1" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="49"/>
+      <c r="C5" s="48"/>
     </row>
     <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="49"/>
+      <c r="C6" s="48"/>
     </row>
     <row r="7" spans="2:3" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
     </row>
     <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="49"/>
+      <c r="C9" s="48"/>
     </row>
     <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
@@ -1859,10 +1869,10 @@
       </c>
     </row>
     <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="51" t="s">
+      <c r="B17" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="49"/>
+      <c r="C17" s="48"/>
     </row>
     <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
@@ -1905,10 +1915,10 @@
       </c>
     </row>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="51" t="s">
+      <c r="B24" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="49"/>
+      <c r="C24" s="48"/>
     </row>
     <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
@@ -1983,10 +1993,10 @@
       </c>
     </row>
     <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="51" t="s">
+      <c r="B36" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="C36" s="49"/>
+      <c r="C36" s="48"/>
     </row>
     <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12" t="s">
@@ -2005,65 +2015,65 @@
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" s="53" t="s">
+      <c r="B41" s="52" t="s">
         <v>50</v>
       </c>
-      <c r="C41" s="49"/>
+      <c r="C41" s="48"/>
     </row>
     <row r="43" spans="2:3" ht="16.5" x14ac:dyDescent="0.3">
       <c r="B43" s="5" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B44" s="59" t="s">
-        <v>283</v>
+      <c r="B44" s="58" t="s">
+        <v>281</v>
       </c>
       <c r="C44" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="58" t="s">
+        <v>322</v>
+      </c>
+      <c r="C45" s="59" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B46" s="58" t="s">
+        <v>323</v>
+      </c>
+      <c r="C46" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="45" spans="2:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="59" t="s">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B47" s="58" t="s">
         <v>325</v>
       </c>
-      <c r="C45" s="60" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B46" s="59" t="s">
+      <c r="C47" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B48" s="58" t="s">
         <v>326</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C48" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" s="58" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B47" s="59" t="s">
+      <c r="C49" t="s">
         <v>328</v>
-      </c>
-      <c r="C47" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B48" s="59" t="s">
-        <v>329</v>
-      </c>
-      <c r="C48" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B49" s="59" t="s">
-        <v>330</v>
-      </c>
-      <c r="C49" t="s">
-        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -2100,8 +2110,8 @@
       </c>
     </row>
     <row r="3" spans="2:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B3" s="47" t="s">
-        <v>319</v>
+      <c r="B3" s="46" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2136,19 +2146,19 @@
       <c r="B7" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="46">
+      <c r="C7" s="45">
         <v>83380686</v>
       </c>
-      <c r="D7" s="46">
+      <c r="D7" s="45">
         <v>51301250</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="G7" s="46">
+      <c r="G7" s="45">
         <v>114000484</v>
       </c>
-      <c r="H7" s="46">
+      <c r="H7" s="45">
         <v>95189145</v>
       </c>
     </row>
@@ -2156,19 +2166,19 @@
       <c r="B8" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="45">
         <v>267209963</v>
       </c>
-      <c r="D8" s="46">
+      <c r="D8" s="45">
         <v>190046565</v>
       </c>
       <c r="F8" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="46">
+      <c r="G8" s="45">
         <v>57785917</v>
       </c>
-      <c r="H8" s="46">
+      <c r="H8" s="45">
         <v>45035056</v>
       </c>
     </row>
@@ -2176,19 +2186,19 @@
       <c r="B9" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="45">
         <v>201580276</v>
       </c>
-      <c r="D9" s="46">
+      <c r="D9" s="45">
         <v>114090183</v>
       </c>
       <c r="F9" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="G9" s="46">
+      <c r="G9" s="45">
         <v>415668163</v>
       </c>
-      <c r="H9" s="46">
+      <c r="H9" s="45">
         <v>365067839</v>
       </c>
     </row>
@@ -2196,10 +2206,10 @@
       <c r="B10" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="45">
         <v>106601539</v>
       </c>
-      <c r="D10" s="46">
+      <c r="D10" s="45">
         <v>41041913</v>
       </c>
       <c r="F10" s="20" t="s">
@@ -2231,10 +2241,10 @@
       <c r="F12" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="G12" s="46">
+      <c r="G12" s="45">
         <v>224500548</v>
       </c>
-      <c r="H12" s="46">
+      <c r="H12" s="45">
         <v>132730912</v>
       </c>
     </row>
@@ -2245,10 +2255,10 @@
       <c r="F13" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G13" s="46">
+      <c r="G13" s="45">
         <v>155178578</v>
       </c>
-      <c r="H13" s="46">
+      <c r="H13" s="45">
         <v>44746470</v>
       </c>
     </row>
@@ -2256,10 +2266,10 @@
       <c r="B14" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="46">
+      <c r="C14" s="45">
         <v>298694616</v>
       </c>
-      <c r="D14" s="46">
+      <c r="D14" s="45">
         <v>258629492</v>
       </c>
     </row>
@@ -2267,10 +2277,10 @@
       <c r="B15" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="46">
+      <c r="C15" s="45">
         <v>103300472</v>
       </c>
-      <c r="D15" s="46">
+      <c r="D15" s="45">
         <v>75686159</v>
       </c>
       <c r="F15" s="20" t="s">
@@ -2310,10 +2320,10 @@
       <c r="F18" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="46">
+      <c r="G18" s="45">
         <v>97211548</v>
       </c>
-      <c r="H18" s="46">
+      <c r="H18" s="45">
         <v>109366131</v>
       </c>
     </row>
@@ -2321,19 +2331,19 @@
       <c r="B19" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="46">
+      <c r="C19" s="45">
         <v>3955994</v>
       </c>
-      <c r="D19" s="46">
+      <c r="D19" s="45">
         <v>4517414</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="46">
+      <c r="G19" s="45">
         <v>54277387</v>
       </c>
-      <c r="H19" s="46">
+      <c r="H19" s="45">
         <v>44468350</v>
       </c>
     </row>
@@ -2341,10 +2351,10 @@
       <c r="B20" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="46">
+      <c r="C20" s="45">
         <v>260500023</v>
       </c>
-      <c r="D20" s="46">
+      <c r="D20" s="45">
         <v>252663245</v>
       </c>
       <c r="F20" s="20" t="s">
@@ -2408,24 +2418,24 @@
     </row>
     <row r="3" spans="2:6" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" s="58" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="56" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" s="57" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="57" t="s">
+      <c r="C5" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="57" t="s">
+      <c r="D5" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="E5" s="55" t="s">
-        <v>322</v>
-      </c>
-      <c r="F5" s="55" t="s">
-        <v>323</v>
+      <c r="E5" s="54" t="s">
+        <v>319</v>
+      </c>
+      <c r="F5" s="54" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2688,17 +2698,17 @@
     </row>
     <row r="3" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="57" t="s">
+      <c r="C5" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="57" t="s">
+      <c r="D5" s="56" t="s">
         <v>54</v>
       </c>
       <c r="E5" s="23" t="s">
@@ -3052,7 +3062,7 @@
         <v>132</v>
       </c>
       <c r="C6" s="29">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D6" s="30"/>
       <c r="E6" s="30" t="s">
@@ -3065,7 +3075,7 @@
       </c>
       <c r="C7" s="31">
         <f>yearCurrent-1</f>
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D7" s="30" t="s">
         <v>135</v>
@@ -3076,407 +3086,411 @@
     </row>
     <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="C8" s="32"/>
+        <v>332</v>
+      </c>
+      <c r="C8" s="60">
+        <v>169600</v>
+      </c>
       <c r="D8" s="30"/>
       <c r="E8" s="30" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="C9" s="33"/>
+        <v>138</v>
+      </c>
+      <c r="C9" s="32">
+        <v>7706</v>
+      </c>
       <c r="D9" s="30"/>
       <c r="E9" s="30" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="C10" s="34">
-        <v>0.09</v>
+        <v>140</v>
+      </c>
+      <c r="C10" s="33">
+        <v>0.12</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="C11" s="34">
-        <v>0.21</v>
+        <v>142</v>
+      </c>
+      <c r="C11" s="33">
+        <v>0.2</v>
       </c>
       <c r="D11" s="30"/>
       <c r="E11" s="30" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="C12" s="34">
+        <f>share_price*shares_outstanding</f>
+        <v>1306937600</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="E12" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="C12" s="35">
-        <f>share_price*shares_outstanding</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="30" t="s">
+    </row>
+    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="53" t="s">
         <v>146</v>
       </c>
-      <c r="E12" s="30" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="54" t="s">
-        <v>148</v>
-      </c>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
     </row>
     <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C15" s="36">
+        <v>147</v>
+      </c>
+      <c r="C15" s="35">
         <f>BAL_equity_shareholders_prior</f>
         <v>153834481</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E15" s="30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="C16" s="36">
+        <v>150</v>
+      </c>
+      <c r="C16" s="35">
         <f>BAL_inventories_prior</f>
         <v>114090183</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="C17" s="36">
+        <v>153</v>
+      </c>
+      <c r="C17" s="35">
         <f>BAL_receivables_prior</f>
         <v>190046565</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="C18" s="36">
+        <v>156</v>
+      </c>
+      <c r="C18" s="35">
         <f>BAL_assets_total_prior</f>
         <v>836603903</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="C19" s="36">
+        <v>159</v>
+      </c>
+      <c r="C19" s="35">
         <f>BAL_debt_long_term_prior+BAL_equity_shareholders_prior</f>
         <v>286565393</v>
       </c>
       <c r="D19" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="E19" s="30" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="53" t="s">
         <v>162</v>
       </c>
-      <c r="E19" s="30" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="54" t="s">
-        <v>164</v>
-      </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
     </row>
     <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="C22" s="35">
+        <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
+        <v>34392602.799999997</v>
+      </c>
+      <c r="D22" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="E22" s="30" t="s">
         <v>165</v>
-      </c>
-      <c r="C22" s="36">
-        <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
-        <v>34101005.439999998</v>
-      </c>
-      <c r="D22" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="C23" s="37">
+        <v>166</v>
+      </c>
+      <c r="C23" s="36">
         <f>IFERROR(INC_sales/365,"")</f>
         <v>909144.00273972598</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E23" s="30" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="C24" s="36">
+        <v>169</v>
+      </c>
+      <c r="C24" s="35">
         <f>BAL_equity_shareholders_curr</f>
         <v>151488935</v>
       </c>
       <c r="D24" s="30" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="C25" s="36">
+        <v>172</v>
+      </c>
+      <c r="C25" s="35">
         <f>BAL_cash_marketable_securities_curr</f>
         <v>83380686</v>
       </c>
       <c r="D25" s="30" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E25" s="30" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="C26" s="36">
+        <v>175</v>
+      </c>
+      <c r="C26" s="35">
         <f>BAL_assets_current_curr</f>
         <v>658772464</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E26" s="30" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="C27" s="36">
+        <v>178</v>
+      </c>
+      <c r="C27" s="35">
         <f>BAL_liabilities_current_curr</f>
         <v>587454564</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="C28" s="37">
+        <v>181</v>
+      </c>
+      <c r="C28" s="36">
         <f>IFERROR(INC_cost_goods_sold/365,"")</f>
         <v>678053.44383561646</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="36">
+      <c r="C29" s="35">
         <f>BAL_debt_long_term_curr</f>
         <v>224500548</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="C30" s="36">
+        <v>186</v>
+      </c>
+      <c r="C30" s="35">
         <f>BAL_assets_current_curr-BAL_liabilities_current_curr</f>
         <v>71317900</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E30" s="30" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="12" t="s">
-        <v>191</v>
-      </c>
-      <c r="C31" s="36">
+        <v>189</v>
+      </c>
+      <c r="C31" s="35">
         <f>BAL_assets_total_curr</f>
         <v>1118622625</v>
       </c>
       <c r="D31" s="30" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E31" s="30" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="C32" s="36">
+        <v>192</v>
+      </c>
+      <c r="C32" s="35">
         <f>BAL_debt_long_term_curr+BAL_equity_shareholders_curr</f>
         <v>375989483</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E32" s="30" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="C33" s="36">
+        <v>195</v>
+      </c>
+      <c r="C33" s="35">
         <f>BAL_liabilities_total_curr</f>
         <v>967133690</v>
       </c>
       <c r="D33" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="E33" s="30" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="53" t="s">
         <v>198</v>
       </c>
-      <c r="E33" s="30" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="54" t="s">
-        <v>200</v>
-      </c>
-      <c r="C35" s="49"/>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="C36" s="37">
+        <v>199</v>
+      </c>
+      <c r="C36" s="36">
         <f>AVERAGE(startYear_equity,currentYear_equity)</f>
         <v>152661708</v>
       </c>
       <c r="D36" s="30" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E36" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="C37" s="37">
+        <v>202</v>
+      </c>
+      <c r="C37" s="36">
         <f>AVERAGE(startYear_total_assets,currentYear_assets_total)</f>
         <v>977613264</v>
       </c>
       <c r="D37" s="30" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E37" s="30" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="12" t="s">
-        <v>207</v>
-      </c>
-      <c r="C38" s="37">
+        <v>205</v>
+      </c>
+      <c r="C38" s="36">
         <f>AVERAGE(startYear_total_capitalization,currentYear_total_capitalization)</f>
         <v>331277438</v>
       </c>
       <c r="D38" s="30" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E38" s="30" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="C41" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="D41" s="23" t="s">
         <v>210</v>
-      </c>
-      <c r="C41" s="23" t="s">
-        <v>211</v>
-      </c>
-      <c r="D41" s="23" t="s">
-        <v>212</v>
       </c>
       <c r="E41" s="23" t="s">
         <v>131</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -3484,37 +3498,37 @@
     </row>
     <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="C43" s="38"/>
+        <v>213</v>
+      </c>
+      <c r="C43" s="37"/>
       <c r="D43" s="30" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E43" s="30"/>
     </row>
     <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="12" t="s">
-        <v>217</v>
-      </c>
-      <c r="C44" s="39"/>
+        <v>215</v>
+      </c>
+      <c r="C44" s="38"/>
       <c r="D44" s="30" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E44" s="30"/>
     </row>
     <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="C45" s="38"/>
+        <v>217</v>
+      </c>
+      <c r="C45" s="37"/>
       <c r="D45" s="30" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E45" s="30"/>
     </row>
     <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -3522,67 +3536,67 @@
     </row>
     <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="C47" s="40"/>
+        <v>220</v>
+      </c>
+      <c r="C47" s="39"/>
       <c r="D47" s="30" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E47" s="30"/>
     </row>
     <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="C48" s="40"/>
+        <v>222</v>
+      </c>
+      <c r="C48" s="39"/>
       <c r="D48" s="30" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E48" s="30"/>
     </row>
     <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="C49" s="40"/>
+        <v>224</v>
+      </c>
+      <c r="C49" s="39"/>
       <c r="D49" s="30" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E49" s="30"/>
     </row>
     <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="C50" s="40"/>
+        <v>226</v>
+      </c>
+      <c r="C50" s="39"/>
       <c r="D50" s="30" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E50" s="30"/>
     </row>
     <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="C51" s="40"/>
+        <v>228</v>
+      </c>
+      <c r="C51" s="39"/>
       <c r="D51" s="30" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E51" s="30"/>
     </row>
     <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="C52" s="40"/>
+        <v>230</v>
+      </c>
+      <c r="C52" s="39"/>
       <c r="D52" s="30" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E52" s="30"/>
     </row>
     <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -3590,81 +3604,81 @@
     </row>
     <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="C54" s="38"/>
+      <c r="D54" s="30" t="s">
+        <v>234</v>
+      </c>
+      <c r="E54" s="30" t="s">
         <v>235</v>
-      </c>
-      <c r="C54" s="39"/>
-      <c r="D54" s="30" t="s">
-        <v>236</v>
-      </c>
-      <c r="E54" s="30" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="C55" s="39"/>
+        <v>236</v>
+      </c>
+      <c r="C55" s="38"/>
       <c r="D55" s="30" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E55" s="30"/>
     </row>
     <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="C56" s="41"/>
+        <v>238</v>
+      </c>
+      <c r="C56" s="40"/>
       <c r="D56" s="30" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E56" s="30"/>
     </row>
     <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="12" t="s">
-        <v>242</v>
-      </c>
-      <c r="C57" s="39"/>
+        <v>240</v>
+      </c>
+      <c r="C57" s="38"/>
       <c r="D57" s="30" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E57" s="30"/>
     </row>
     <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="C58" s="41"/>
+        <v>242</v>
+      </c>
+      <c r="C58" s="40"/>
       <c r="D58" s="30" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E58" s="30"/>
     </row>
     <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="C59" s="40"/>
+        <v>244</v>
+      </c>
+      <c r="C59" s="39"/>
       <c r="D59" s="30" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E59" s="30"/>
     </row>
     <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="C60" s="39"/>
+      <c r="D60" s="30" t="s">
+        <v>247</v>
+      </c>
+      <c r="E60" s="30" t="s">
         <v>248</v>
-      </c>
-      <c r="C60" s="40"/>
-      <c r="D60" s="30" t="s">
-        <v>249</v>
-      </c>
-      <c r="E60" s="30" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -3672,81 +3686,81 @@
     </row>
     <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="12" t="s">
-        <v>252</v>
-      </c>
-      <c r="C62" s="40"/>
+        <v>250</v>
+      </c>
+      <c r="C62" s="39"/>
       <c r="D62" s="30" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E62" s="30"/>
     </row>
     <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="C63" s="39"/>
+        <v>252</v>
+      </c>
+      <c r="C63" s="38"/>
       <c r="D63" s="30" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E63" s="30"/>
     </row>
     <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="12" t="s">
-        <v>256</v>
-      </c>
-      <c r="C64" s="40"/>
+        <v>254</v>
+      </c>
+      <c r="C64" s="39"/>
       <c r="D64" s="30" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E64" s="30"/>
     </row>
     <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="12" t="s">
-        <v>258</v>
-      </c>
-      <c r="C65" s="39"/>
+        <v>256</v>
+      </c>
+      <c r="C65" s="38"/>
       <c r="D65" s="30" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E65" s="30"/>
     </row>
     <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="C66" s="39"/>
+        <v>258</v>
+      </c>
+      <c r="C66" s="38"/>
       <c r="D66" s="30" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E66" s="30"/>
     </row>
     <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="C67" s="41"/>
+      <c r="D67" s="30" t="s">
+        <v>261</v>
+      </c>
+      <c r="E67" s="30" t="s">
         <v>262</v>
-      </c>
-      <c r="C67" s="42"/>
-      <c r="D67" s="30" t="s">
-        <v>263</v>
-      </c>
-      <c r="E67" s="30" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="C68" s="38"/>
+      <c r="D68" s="30" t="s">
+        <v>264</v>
+      </c>
+      <c r="E68" s="30" t="s">
         <v>265</v>
-      </c>
-      <c r="C68" s="39"/>
-      <c r="D68" s="30" t="s">
-        <v>266</v>
-      </c>
-      <c r="E68" s="30" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -3754,47 +3768,47 @@
     </row>
     <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="C70" s="40"/>
+        <v>267</v>
+      </c>
+      <c r="C70" s="39"/>
       <c r="D70" s="30" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="E70" s="30"/>
     </row>
     <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="C71" s="39"/>
+        <v>269</v>
+      </c>
+      <c r="C71" s="38"/>
       <c r="D71" s="30" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E71" s="30"/>
     </row>
     <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="C72" s="39"/>
+        <v>271</v>
+      </c>
+      <c r="C72" s="38"/>
       <c r="D72" s="30" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E72" s="30"/>
     </row>
     <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="12" t="s">
-        <v>275</v>
-      </c>
-      <c r="C73" s="39"/>
+        <v>273</v>
+      </c>
+      <c r="C73" s="38"/>
       <c r="D73" s="30" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E73" s="30"/>
     </row>
     <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -3802,25 +3816,25 @@
     </row>
     <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="C75" s="40"/>
+        <v>276</v>
+      </c>
+      <c r="C75" s="39"/>
       <c r="D75" s="30" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E75" s="30"/>
-      <c r="F75" s="44" t="str">
+      <c r="F75" s="43" t="str">
         <f>IF(OR(C75="",C47=""),"",IF(ROUND(C75,6)=ROUND(C47,6),"✓ matches direct ROA","✗ differs by "&amp;TEXT(ABS(C75-C47),"0.00%")))</f>
         <v/>
       </c>
     </row>
     <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="12" t="s">
-        <v>280</v>
-      </c>
-      <c r="C76" s="40"/>
+        <v>278</v>
+      </c>
+      <c r="C76" s="39"/>
       <c r="D76" s="30" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E76" s="30"/>
     </row>
@@ -3846,156 +3860,156 @@
   <sheetData>
     <row r="2" spans="2:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="14" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="42" t="s">
+        <v>281</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="43" t="s">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="42" t="s">
         <v>283</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="43" t="s">
+    <row r="6" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="42" t="s">
         <v>285</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C6" s="44" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="42" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="43" t="s">
+      <c r="C7" s="44" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="42" t="s">
         <v>287</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C8" s="44" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="B9" s="42" t="s">
+        <v>288</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B10" s="42" t="s">
+        <v>289</v>
+      </c>
+      <c r="C10" s="44" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="43" t="s">
-        <v>288</v>
-      </c>
-      <c r="C7" s="45" t="s">
+    <row r="11" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B11" s="42" t="s">
+        <v>290</v>
+      </c>
+      <c r="C11" s="44" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="43" t="s">
-        <v>289</v>
-      </c>
-      <c r="C8" s="45" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="B9" s="43" t="s">
-        <v>290</v>
-      </c>
-      <c r="C9" s="45" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B10" s="43" t="s">
+    <row r="12" spans="2:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="B12" s="42" t="s">
         <v>291</v>
       </c>
-      <c r="C10" s="45" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B11" s="43" t="s">
+      <c r="C12" s="44" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B13" s="42" t="s">
         <v>292</v>
       </c>
-      <c r="C11" s="45" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="B12" s="43" t="s">
+      <c r="C13" s="44" t="s">
         <v>293</v>
       </c>
-      <c r="C12" s="45" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="13" spans="2:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B13" s="43" t="s">
+    </row>
+    <row r="14" spans="2:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="B14" s="42" t="s">
         <v>294</v>
       </c>
-      <c r="C13" s="45" t="s">
+      <c r="C14" s="44" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="42" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="14" spans="2:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="B14" s="43" t="s">
+      <c r="C15" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="C14" s="45" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="43" t="s">
+    </row>
+    <row r="16" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="42" t="s">
         <v>297</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="16" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="43" t="s">
+    <row r="17" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="42" t="s">
         <v>299</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="43" t="s">
+    <row r="18" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="42" t="s">
         <v>301</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="43" t="s">
+    <row r="19" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="42" t="s">
         <v>303</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="43" t="s">
+    <row r="20" spans="2:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="42" t="s">
         <v>305</v>
       </c>
-      <c r="C19" s="4" t="s">
+    </row>
+    <row r="21" spans="2:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="42" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="20" spans="2:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="43" t="s">
+      <c r="C21" s="4" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="43" t="s">
+    <row r="22" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
         <v>308</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>309</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="43" t="s">
-        <v>310</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update the file format and submit the assignment at Stage 3
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-22-tran-vingroup-financials.xlsx
+++ b/models/builds/2026-05-22-tran-vingroup-financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tan\Leanings\VEMBA Hawaii\Corporate_Finance\Corporate-Finance\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AEC2B0E-D590-48BD-866D-C2296869B154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75EBADF6-F83C-4511-A3EC-CE5210808250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22185" yWindow="2610" windowWidth="13860" windowHeight="27600" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13890" yWindow="2820" windowWidth="37725" windowHeight="27600" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="330">
   <si>
     <t>UNIVERSITY OF HAWAIʻI AT MĀNOA · SHIDLER COLLEGE OF BUSINESS</t>
   </si>
@@ -135,9 +135,6 @@
     <t>BUS-629 International Corporate Finance · Vietnam EMBA</t>
   </si>
   <si>
-    <t>Performance Ratios — Excel Template</t>
-  </si>
-  <si>
     <t>How to Use This Template</t>
   </si>
   <si>
@@ -262,24 +259,6 @@
   </si>
   <si>
     <t>Key ratios reused in Du Pont decomposition (asset_turnover, operating_profit_margin, leverage, debt_burden).</t>
-  </si>
-  <si>
-    <t>Companion Specification</t>
-  </si>
-  <si>
-    <t>See:</t>
-  </si>
-  <si>
-    <t>docs/templates/spec-template.md (repo-level)</t>
-  </si>
-  <si>
-    <t>Course:</t>
-  </si>
-  <si>
-    <t>courses/BUS-629-VEMBA-International-Corporate-Finance/</t>
-  </si>
-  <si>
-    <t>Prepared per UH Mānoa brand standards (docs/_branding/design.json). Primary green #024731 · Open Sans typography · ADA-compliant contrast.</t>
   </si>
   <si>
     <t>Balance Sheet</t>
@@ -1139,6 +1118,12 @@
   </si>
   <si>
     <t>Market capitalization (VND million)</t>
+  </si>
+  <si>
+    <t>Performance Ratios</t>
+  </si>
+  <si>
+    <t>Cover</t>
   </si>
 </sst>
 </file>
@@ -1150,13 +1135,13 @@
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;—&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\);&quot;—&quot;"/>
-    <numFmt numFmtId="168" formatCode="#,##0.00;\(#,##0.00\);&quot;—&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="170" formatCode="0.0&quot; days&quot;"/>
-    <numFmt numFmtId="171" formatCode="0.000"/>
-    <numFmt numFmtId="177" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00;\(#,##0.00\);&quot;—&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot; days&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="171" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1226,12 +1211,6 @@
       <color rgb="FF525252"/>
       <name val="Consolas"/>
       <family val="3"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="8"/>
-      <color rgb="FF525252"/>
-      <name val="Open Sans"/>
     </font>
     <font>
       <b/>
@@ -1338,7 +1317,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1361,12 +1340,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1396,9 +1390,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1415,50 +1408,35 @@
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="170" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1471,11 +1449,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="8" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1779,7 +1781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:C49"/>
+  <dimension ref="B2:C42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1793,297 +1795,275 @@
       <c r="C2" s="1"/>
     </row>
     <row r="4" spans="2:3" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B4" s="47" t="s">
+      <c r="B4" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="48"/>
+      <c r="C4" s="52"/>
     </row>
     <row r="5" spans="2:3" ht="26.1" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="51" t="s">
+      <c r="B5" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="48"/>
+      <c r="C5" s="52"/>
     </row>
     <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="49" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="48"/>
+      <c r="B6" s="53" t="s">
+        <v>328</v>
+      </c>
+      <c r="C6" s="52"/>
     </row>
     <row r="7" spans="2:3" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
     </row>
-    <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="50" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="48"/>
+    <row r="8" spans="2:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="54" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="52"/>
     </row>
     <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>4</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="4" t="s">
+    </row>
+    <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="54" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="48"/>
+      <c r="C17" s="52"/>
     </row>
     <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="7" t="s">
+    </row>
+    <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="54" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="48"/>
+      <c r="C24" s="52"/>
     </row>
     <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="7" t="s">
         <v>33</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" s="7" t="s">
         <v>35</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>39</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="50" t="s">
-        <v>45</v>
-      </c>
-      <c r="C36" s="48"/>
-    </row>
-    <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>49</v>
+    </row>
+    <row r="35" spans="2:3" ht="18.75" x14ac:dyDescent="0.35">
+      <c r="B35" s="54" t="s">
+        <v>329</v>
+      </c>
+      <c r="C35" s="52"/>
+    </row>
+    <row r="36" spans="2:3" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="B36" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="48" t="s">
+        <v>274</v>
+      </c>
+      <c r="C37" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="57" t="s">
+        <v>315</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B39" s="48" t="s">
+        <v>316</v>
+      </c>
+      <c r="C39" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B40" s="48" t="s">
+        <v>318</v>
+      </c>
+      <c r="C40" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" s="52" t="s">
-        <v>50</v>
-      </c>
-      <c r="C41" s="48"/>
-    </row>
-    <row r="43" spans="2:3" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B43" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B44" s="58" t="s">
-        <v>281</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="B41" s="48" t="s">
+        <v>319</v>
+      </c>
+      <c r="C41" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B42" s="48" t="s">
+        <v>320</v>
+      </c>
+      <c r="C42" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="45" spans="2:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="58" t="s">
-        <v>322</v>
-      </c>
-      <c r="C45" s="59" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B46" s="58" t="s">
-        <v>323</v>
-      </c>
-      <c r="C46" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B47" s="58" t="s">
-        <v>325</v>
-      </c>
-      <c r="C47" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B48" s="58" t="s">
-        <v>326</v>
-      </c>
-      <c r="C48" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B49" s="58" t="s">
-        <v>327</v>
-      </c>
-      <c r="C49" t="s">
-        <v>328</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="7">
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B9:C9"/>
   </mergeCells>
@@ -2105,266 +2085,266 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="14" t="s">
-        <v>51</v>
+      <c r="B2" s="13" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B3" s="46" t="s">
-        <v>316</v>
+      <c r="B3" s="43" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>54</v>
+      <c r="B5" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>57</v>
+      <c r="B6" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="45">
+        <v>51</v>
+      </c>
+      <c r="C7" s="42">
         <v>83380686</v>
       </c>
-      <c r="D7" s="45">
+      <c r="D7" s="42">
         <v>51301250</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7" s="45">
+        <v>52</v>
+      </c>
+      <c r="G7" s="42">
         <v>114000484</v>
       </c>
-      <c r="H7" s="45">
+      <c r="H7" s="42">
         <v>95189145</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" s="45">
+        <v>53</v>
+      </c>
+      <c r="C8" s="42">
         <v>267209963</v>
       </c>
-      <c r="D8" s="45">
+      <c r="D8" s="42">
         <v>190046565</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="45">
+        <v>54</v>
+      </c>
+      <c r="G8" s="42">
         <v>57785917</v>
       </c>
-      <c r="H8" s="45">
+      <c r="H8" s="42">
         <v>45035056</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="45">
+        <v>55</v>
+      </c>
+      <c r="C9" s="42">
         <v>201580276</v>
       </c>
-      <c r="D9" s="45">
+      <c r="D9" s="42">
         <v>114090183</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="G9" s="45">
+        <v>56</v>
+      </c>
+      <c r="G9" s="42">
         <v>415668163</v>
       </c>
-      <c r="H9" s="45">
+      <c r="H9" s="42">
         <v>365067839</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="45">
+        <v>57</v>
+      </c>
+      <c r="C10" s="42">
         <v>106601539</v>
       </c>
-      <c r="D10" s="45">
+      <c r="D10" s="42">
         <v>41041913</v>
       </c>
-      <c r="F10" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="G10" s="21">
+      <c r="F10" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="20">
         <f>SUM(G7:G9)</f>
         <v>587454564</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="20">
         <f>SUM(H7:H9)</f>
         <v>505292040</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="21">
+      <c r="B11" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="20">
         <f>SUM(C7:C10)</f>
         <v>658772464</v>
       </c>
-      <c r="D11" s="21">
+      <c r="D11" s="20">
         <f>SUM(D7:D10)</f>
         <v>396479911</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F12" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="G12" s="45">
+        <v>60</v>
+      </c>
+      <c r="G12" s="42">
         <v>224500548</v>
       </c>
-      <c r="H12" s="45">
+      <c r="H12" s="42">
         <v>132730912</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="18" t="s">
-        <v>68</v>
+      <c r="B13" s="17" t="s">
+        <v>61</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="G13" s="45">
+        <v>62</v>
+      </c>
+      <c r="G13" s="42">
         <v>155178578</v>
       </c>
-      <c r="H13" s="45">
+      <c r="H13" s="42">
         <v>44746470</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="45">
+        <v>63</v>
+      </c>
+      <c r="C14" s="42">
         <v>298694616</v>
       </c>
-      <c r="D14" s="45">
+      <c r="D14" s="42">
         <v>258629492</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="45">
+        <v>64</v>
+      </c>
+      <c r="C15" s="42">
         <v>103300472</v>
       </c>
-      <c r="D15" s="45">
+      <c r="D15" s="42">
         <v>75686159</v>
       </c>
-      <c r="F15" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="G15" s="21">
+      <c r="F15" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="20">
         <f>G10+G12+G13</f>
         <v>967133690</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="20">
         <f>H10+H12+H13</f>
         <v>682769422</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="21">
+      <c r="B16" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="20">
         <f>C14-C15</f>
         <v>195394144</v>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="20">
         <f>D14-D15</f>
         <v>182943333</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F17" s="18" t="s">
-        <v>74</v>
+      <c r="F17" s="17" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="18" t="s">
-        <v>75</v>
+      <c r="B18" s="17" t="s">
+        <v>68</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="G18" s="45">
+        <v>69</v>
+      </c>
+      <c r="G18" s="42">
         <v>97211548</v>
       </c>
-      <c r="H18" s="45">
+      <c r="H18" s="42">
         <v>109366131</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="C19" s="45">
+        <v>70</v>
+      </c>
+      <c r="C19" s="42">
         <v>3955994</v>
       </c>
-      <c r="D19" s="45">
+      <c r="D19" s="42">
         <v>4517414</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="G19" s="45">
+        <v>71</v>
+      </c>
+      <c r="G19" s="42">
         <v>54277387</v>
       </c>
-      <c r="H19" s="45">
+      <c r="H19" s="42">
         <v>44468350</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="C20" s="45">
+        <v>72</v>
+      </c>
+      <c r="C20" s="42">
         <v>260500023</v>
       </c>
-      <c r="D20" s="45">
+      <c r="D20" s="42">
         <v>252663245</v>
       </c>
-      <c r="F20" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="G20" s="21">
+      <c r="F20" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="G20" s="20">
         <f>G18+G19</f>
         <v>151488935</v>
       </c>
-      <c r="H20" s="21">
+      <c r="H20" s="20">
         <f>H18+H19</f>
         <v>153834481</v>
       </c>
@@ -2372,24 +2352,24 @@
     <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C23" s="22">
+        <v>74</v>
+      </c>
+      <c r="C23" s="21">
         <f>C11+C16+C19+C20</f>
         <v>1118622625</v>
       </c>
-      <c r="D23" s="22">
+      <c r="D23" s="21">
         <f>D11+D16+D19+D20</f>
         <v>836603903</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G23" s="22">
+        <v>75</v>
+      </c>
+      <c r="G23" s="21">
         <f>G15+G20</f>
         <v>1118622625</v>
       </c>
-      <c r="H23" s="22">
+      <c r="H23" s="21">
         <f>H15+H20</f>
         <v>836603903</v>
       </c>
@@ -2412,265 +2392,265 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="14" t="s">
-        <v>83</v>
+      <c r="B2" s="13" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B3" s="15" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" s="57" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="55" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="56" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="56" t="s">
-        <v>54</v>
-      </c>
-      <c r="E5" s="54" t="s">
-        <v>319</v>
-      </c>
-      <c r="F5" s="54" t="s">
-        <v>320</v>
+      <c r="B3" s="14" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" s="47" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="45" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>312</v>
+      </c>
+      <c r="F5" s="44" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="C6" s="19">
+        <v>78</v>
+      </c>
+      <c r="C6" s="18">
         <v>331837561</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="18">
         <v>189068040</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="23">
         <v>1</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="23">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="C7" s="19">
+        <v>79</v>
+      </c>
+      <c r="C7" s="18">
         <v>247489507</v>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="18">
         <v>139140098</v>
       </c>
-      <c r="E7" s="25">
-        <f>IFERROR(C7/$C$6,"")</f>
+      <c r="E7" s="24">
+        <f t="shared" ref="E7:E15" si="0">IFERROR(C7/$C$6,"")</f>
         <v>0.74581523036206265</v>
       </c>
-      <c r="F7" s="25">
+      <c r="F7" s="24">
         <f>IFERROR(D7/$D$6,"")</f>
         <v>0.73592606132691707</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C8" s="19">
+        <v>80</v>
+      </c>
+      <c r="C8" s="18">
         <v>49053914</v>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="18">
         <v>33202226</v>
       </c>
-      <c r="E8" s="25">
-        <f>IFERROR(C8/$C$6,"")</f>
+      <c r="E8" s="24">
+        <f t="shared" si="0"/>
         <v>0.1478250799944856</v>
       </c>
-      <c r="F8" s="25">
-        <f t="shared" ref="F8:F14" si="0">IFERROR(D8/$D$6,"")</f>
+      <c r="F8" s="24">
+        <f t="shared" ref="F8:F14" si="1">IFERROR(D8/$D$6,"")</f>
         <v>0.17560993386296278</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="C9" s="19">
+        <v>81</v>
+      </c>
+      <c r="C9" s="18">
         <v>31665247</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="18">
         <v>22627124</v>
       </c>
-      <c r="E9" s="25">
-        <f>IFERROR(C9/$C$6,"")</f>
+      <c r="E9" s="24">
+        <f t="shared" si="0"/>
         <v>9.5423938461264179E-2</v>
       </c>
-      <c r="F9" s="25">
-        <f t="shared" si="0"/>
+      <c r="F9" s="24">
+        <f t="shared" si="1"/>
         <v>0.1196771490305818</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="C10" s="21">
+      <c r="B10" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="20">
         <f>C6-C7-C8-C9</f>
         <v>3628893</v>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="20">
         <f>D6-D7-D8-D9</f>
         <v>-5901408</v>
       </c>
-      <c r="E10" s="25">
-        <f>IFERROR(C10/$C$6,"")</f>
+      <c r="E10" s="24">
+        <f t="shared" si="0"/>
         <v>1.0935751182187601E-2</v>
       </c>
-      <c r="F10" s="25">
-        <f t="shared" si="0"/>
+      <c r="F10" s="24">
+        <f t="shared" si="1"/>
         <v>-3.1213144220461585E-2</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" s="19">
+        <v>83</v>
+      </c>
+      <c r="C11" s="18">
         <v>51968218</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="18">
         <v>45620158</v>
       </c>
-      <c r="E11" s="25">
-        <f>IFERROR(C11/$C$6,"")</f>
+      <c r="E11" s="24">
+        <f t="shared" si="0"/>
         <v>0.15660740105307128</v>
       </c>
-      <c r="F11" s="25">
-        <f t="shared" si="0"/>
+      <c r="F11" s="24">
+        <f t="shared" si="1"/>
         <v>0.24128963308658619</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C12" s="19">
+        <v>84</v>
+      </c>
+      <c r="C12" s="18">
         <v>29159736</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="18">
         <v>22980044</v>
       </c>
-      <c r="E12" s="25">
-        <f>IFERROR(C12/$C$6,"")</f>
+      <c r="E12" s="24">
+        <f t="shared" si="0"/>
         <v>8.7873524359709243E-2</v>
       </c>
-      <c r="F12" s="25">
-        <f t="shared" si="0"/>
+      <c r="F12" s="24">
+        <f t="shared" si="1"/>
         <v>0.12154377863122715</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="C13" s="21">
+      <c r="B13" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="20">
         <f>C10+C11-C12</f>
         <v>26437375</v>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="20">
         <f>D10+D11-D12</f>
         <v>16738706</v>
       </c>
-      <c r="E13" s="25">
-        <f>IFERROR(C13/$C$6,"")</f>
+      <c r="E13" s="24">
+        <f t="shared" si="0"/>
         <v>7.9669627875549626E-2</v>
       </c>
-      <c r="F13" s="25">
-        <f t="shared" si="0"/>
+      <c r="F13" s="24">
+        <f t="shared" si="1"/>
         <v>8.8532710234897449E-2</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="C14" s="19">
+        <v>86</v>
+      </c>
+      <c r="C14" s="18">
         <v>15372561</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="18">
         <v>11462648</v>
       </c>
-      <c r="E14" s="25">
-        <f>IFERROR(C14/$C$6,"")</f>
+      <c r="E14" s="24">
+        <f t="shared" si="0"/>
         <v>4.6325560475054241E-2</v>
       </c>
-      <c r="F14" s="25">
-        <f t="shared" si="0"/>
+      <c r="F14" s="24">
+        <f t="shared" si="1"/>
         <v>6.0627105458965991E-2</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="C15" s="22">
+        <v>87</v>
+      </c>
+      <c r="C15" s="21">
         <f>C13-C14</f>
         <v>11064814</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="21">
         <f>D13-D14</f>
         <v>5276058</v>
       </c>
-      <c r="E15" s="26">
-        <f>IFERROR(C15/$C$6,"")</f>
+      <c r="E15" s="25">
+        <f t="shared" si="0"/>
         <v>3.3344067400495392E-2</v>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="25">
         <f>IFERROR(D15/$D$6,"")</f>
         <v>2.7905604775931458E-2</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="18" t="s">
-        <v>95</v>
+      <c r="B17" s="17" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19">
+        <v>89</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18">
         <v>666188</v>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="24">
         <f>IFERROR(C18/$C$6,"")</f>
         <v>0</v>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="24">
         <f>IFERROR(D18/$D$6,"")</f>
         <v>3.5235357599306578E-3</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="C19" s="21">
+      <c r="B19" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" s="20">
         <f>C15-C18</f>
         <v>11064814</v>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="20">
         <f>D15-D18</f>
         <v>4609870</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="24">
         <f>IFERROR(C19/$C$6,"")</f>
         <v>3.3344067400495392E-2</v>
       </c>
-      <c r="F19" s="25">
+      <c r="F19" s="24">
         <f>IFERROR(D19/$D$6,"")</f>
         <v>2.4382069016000801E-2</v>
       </c>
@@ -2692,328 +2672,328 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="14" t="s">
-        <v>98</v>
+      <c r="B2" s="13" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B3" s="15" t="s">
-        <v>318</v>
+      <c r="B3" s="14" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="56" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="56" t="s">
-        <v>54</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>99</v>
+      <c r="B5" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="E6" s="15"/>
+      <c r="B6" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7" s="27">
+        <v>94</v>
+      </c>
+      <c r="C7" s="26">
         <f>INC_net</f>
         <v>11064814</v>
       </c>
-      <c r="D7" s="27">
+      <c r="D7" s="26">
         <v>5276058</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>102</v>
+      <c r="E7" s="14" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="27">
+        <v>96</v>
+      </c>
+      <c r="C8" s="26">
         <f>INC_depreciation</f>
         <v>31665247</v>
       </c>
-      <c r="D8" s="27">
+      <c r="D8" s="26">
         <v>22627124</v>
       </c>
-      <c r="E8" s="15" t="s">
-        <v>102</v>
+      <c r="E8" s="14" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="E9" s="15"/>
+      <c r="B9" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C10" s="19">
+        <v>98</v>
+      </c>
+      <c r="C10" s="18">
         <v>-20235943</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="18">
         <v>-95017737</v>
       </c>
-      <c r="E10" s="15" t="s">
-        <v>106</v>
+      <c r="E10" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" s="19">
+        <v>100</v>
+      </c>
+      <c r="C11" s="18">
         <v>-67530856</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="18">
         <v>-23011001</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>106</v>
+      <c r="E11" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C12" s="19">
+        <v>101</v>
+      </c>
+      <c r="C12" s="18">
         <v>3985858</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="18">
         <v>-3116968</v>
       </c>
-      <c r="E12" s="15" t="s">
-        <v>106</v>
+      <c r="E12" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C13" s="19">
+        <v>102</v>
+      </c>
+      <c r="C13" s="18">
         <v>12750861</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="18">
         <v>10160792</v>
       </c>
-      <c r="E13" s="15" t="s">
-        <v>106</v>
+      <c r="E13" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="C14" s="19">
+        <v>103</v>
+      </c>
+      <c r="C14" s="18">
         <v>97154801</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="18">
         <v>99548789</v>
       </c>
-      <c r="E14" s="15" t="s">
-        <v>106</v>
+      <c r="E14" s="14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="C15" s="21">
+      <c r="B15" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="20">
         <f>SUM(C10:C14)</f>
         <v>26124721</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="20">
         <f>SUM(D10:D14)</f>
         <v>-11436125</v>
       </c>
-      <c r="E15" s="15"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="16" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="22">
+        <v>105</v>
+      </c>
+      <c r="C16" s="21">
         <f>C7+C8+C15</f>
         <v>68854782</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="21">
         <f>D7+D8+D15</f>
         <v>16467057</v>
       </c>
-      <c r="E16" s="15"/>
+      <c r="E16" s="14"/>
     </row>
     <row r="17" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="E17" s="15"/>
+      <c r="E17" s="14"/>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="E18" s="15"/>
+      <c r="B18" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="E18" s="14"/>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="C19" s="19">
+        <v>107</v>
+      </c>
+      <c r="C19" s="18">
         <v>-76157072</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="18">
         <v>-48567437</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="14"/>
     </row>
     <row r="20" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="C20" s="19">
+        <v>108</v>
+      </c>
+      <c r="C20" s="18">
         <v>65772180</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="18">
         <v>84186330</v>
       </c>
-      <c r="E20" s="15"/>
+      <c r="E20" s="14"/>
     </row>
     <row r="21" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="C21" s="19">
+        <v>109</v>
+      </c>
+      <c r="C21" s="18">
         <v>-129543511</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="18">
         <v>-52461980</v>
       </c>
-      <c r="E21" s="15"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="C22" s="22">
+        <v>110</v>
+      </c>
+      <c r="C22" s="21">
         <f>SUM(C19:C21)</f>
         <v>-139928403</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="21">
         <f>SUM(D19:D21)</f>
         <v>-16843087</v>
       </c>
-      <c r="E22" s="15"/>
+      <c r="E22" s="14"/>
     </row>
     <row r="23" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="E23" s="15"/>
+      <c r="E23" s="14"/>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="E24" s="15"/>
+      <c r="B24" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="E24" s="14"/>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="C25" s="19">
+        <v>112</v>
+      </c>
+      <c r="C25" s="18">
         <v>18811339</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="18">
         <v>-21046056</v>
       </c>
-      <c r="E25" s="15"/>
+      <c r="E25" s="14"/>
     </row>
     <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="C26" s="19">
+        <v>113</v>
+      </c>
+      <c r="C26" s="18">
         <v>83383279</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="18">
         <v>27601580</v>
       </c>
-      <c r="E26" s="15"/>
+      <c r="E26" s="14"/>
     </row>
     <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="C27" s="19">
+        <v>114</v>
+      </c>
+      <c r="C27" s="18">
         <v>-2577141</v>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="18">
         <v>-666188</v>
       </c>
-      <c r="E27" s="15"/>
+      <c r="E27" s="14"/>
     </row>
     <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C28" s="19">
+        <v>115</v>
+      </c>
+      <c r="C28" s="18">
         <v>2267028</v>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="18">
         <v>15659006</v>
       </c>
-      <c r="E28" s="15"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C29" s="19">
+        <v>116</v>
+      </c>
+      <c r="C29" s="18">
         <f>-265382+390107</f>
         <v>124725</v>
       </c>
-      <c r="D29" s="19">
+      <c r="D29" s="18">
         <v>-6234548</v>
       </c>
-      <c r="E29" s="15"/>
+      <c r="E29" s="14"/>
     </row>
     <row r="30" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="C30" s="22">
+        <v>117</v>
+      </c>
+      <c r="C30" s="21">
         <f>SUM(C25:C29)</f>
         <v>102009230</v>
       </c>
-      <c r="D30" s="22">
+      <c r="D30" s="21">
         <f>SUM(D25:D29)</f>
         <v>15313794</v>
       </c>
-      <c r="E30" s="15"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="E31" s="15"/>
+      <c r="E31" s="14"/>
     </row>
     <row r="32" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C32" s="22">
+        <v>118</v>
+      </c>
+      <c r="C32" s="21">
         <f>C16+C22+C30</f>
         <v>30935609</v>
       </c>
-      <c r="D32" s="22">
+      <c r="D32" s="21">
         <f>D16+D22+D30</f>
         <v>14937764</v>
       </c>
-      <c r="E32" s="15"/>
+      <c r="E32" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3034,463 +3014,463 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="14" t="s">
-        <v>126</v>
+      <c r="B2" s="13" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B3" s="15" t="s">
-        <v>127</v>
+      <c r="B3" s="14" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>131</v>
+      <c r="B5" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C6" s="29">
+        <v>125</v>
+      </c>
+      <c r="C6" s="28">
         <v>2025</v>
       </c>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30" t="s">
-        <v>133</v>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="31">
+        <v>127</v>
+      </c>
+      <c r="C7" s="30">
         <f>yearCurrent-1</f>
         <v>2024</v>
       </c>
-      <c r="D7" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="E7" s="30" t="s">
-        <v>136</v>
+      <c r="D7" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="E7" s="29" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>332</v>
-      </c>
-      <c r="C8" s="60">
+        <v>325</v>
+      </c>
+      <c r="C8" s="50">
         <v>169600</v>
       </c>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30" t="s">
-        <v>137</v>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="C9" s="32">
+        <v>131</v>
+      </c>
+      <c r="C9" s="31">
         <v>7706</v>
       </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30" t="s">
-        <v>139</v>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" s="33">
+        <v>133</v>
+      </c>
+      <c r="C10" s="32">
         <v>0.12</v>
       </c>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30" t="s">
-        <v>141</v>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C11" s="33">
+        <v>135</v>
+      </c>
+      <c r="C11" s="32">
         <v>0.2</v>
       </c>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30" t="s">
-        <v>143</v>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
-        <v>334</v>
-      </c>
-      <c r="C12" s="34">
+        <v>327</v>
+      </c>
+      <c r="C12" s="33">
         <f>share_price*shares_outstanding</f>
         <v>1306937600</v>
       </c>
-      <c r="D12" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>145</v>
+      <c r="D12" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="53" t="s">
-        <v>146</v>
-      </c>
-      <c r="C14" s="48"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="48"/>
+      <c r="B14" s="56" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" s="52"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="52"/>
     </row>
     <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="C15" s="35">
+        <v>140</v>
+      </c>
+      <c r="C15" s="34">
         <f>BAL_equity_shareholders_prior</f>
         <v>153834481</v>
       </c>
-      <c r="D15" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>149</v>
+      <c r="D15" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="C16" s="35">
+        <v>143</v>
+      </c>
+      <c r="C16" s="34">
         <f>BAL_inventories_prior</f>
         <v>114090183</v>
       </c>
-      <c r="D16" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>152</v>
+      <c r="D16" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="C17" s="35">
+        <v>146</v>
+      </c>
+      <c r="C17" s="34">
         <f>BAL_receivables_prior</f>
         <v>190046565</v>
       </c>
-      <c r="D17" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>155</v>
+      <c r="D17" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="C18" s="35">
+        <v>149</v>
+      </c>
+      <c r="C18" s="34">
         <f>BAL_assets_total_prior</f>
         <v>836603903</v>
       </c>
-      <c r="D18" s="30" t="s">
-        <v>157</v>
-      </c>
-      <c r="E18" s="30" t="s">
-        <v>158</v>
+      <c r="D18" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="C19" s="35">
+        <v>152</v>
+      </c>
+      <c r="C19" s="34">
         <f>BAL_debt_long_term_prior+BAL_equity_shareholders_prior</f>
         <v>286565393</v>
       </c>
-      <c r="D19" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>161</v>
+      <c r="D19" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="E19" s="29" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="53" t="s">
-        <v>162</v>
-      </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
+      <c r="B21" s="56" t="s">
+        <v>155</v>
+      </c>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
     </row>
     <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="C22" s="35">
+        <v>156</v>
+      </c>
+      <c r="C22" s="34">
         <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
         <v>34392602.799999997</v>
       </c>
-      <c r="D22" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>165</v>
+      <c r="D22" s="29" t="s">
+        <v>157</v>
+      </c>
+      <c r="E22" s="29" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="C23" s="36">
+        <v>159</v>
+      </c>
+      <c r="C23" s="35">
         <f>IFERROR(INC_sales/365,"")</f>
         <v>909144.00273972598</v>
       </c>
-      <c r="D23" s="30" t="s">
-        <v>167</v>
-      </c>
-      <c r="E23" s="30" t="s">
-        <v>168</v>
+      <c r="D23" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="E23" s="29" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="C24" s="35">
+        <v>162</v>
+      </c>
+      <c r="C24" s="34">
         <f>BAL_equity_shareholders_curr</f>
         <v>151488935</v>
       </c>
-      <c r="D24" s="30" t="s">
-        <v>170</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>171</v>
+      <c r="D24" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="E24" s="29" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="C25" s="35">
+        <v>165</v>
+      </c>
+      <c r="C25" s="34">
         <f>BAL_cash_marketable_securities_curr</f>
         <v>83380686</v>
       </c>
-      <c r="D25" s="30" t="s">
-        <v>173</v>
-      </c>
-      <c r="E25" s="30" t="s">
-        <v>174</v>
+      <c r="D25" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="C26" s="35">
+        <v>168</v>
+      </c>
+      <c r="C26" s="34">
         <f>BAL_assets_current_curr</f>
         <v>658772464</v>
       </c>
-      <c r="D26" s="30" t="s">
-        <v>176</v>
-      </c>
-      <c r="E26" s="30" t="s">
-        <v>177</v>
+      <c r="D26" s="29" t="s">
+        <v>169</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="C27" s="35">
+        <v>171</v>
+      </c>
+      <c r="C27" s="34">
         <f>BAL_liabilities_current_curr</f>
         <v>587454564</v>
       </c>
-      <c r="D27" s="30" t="s">
-        <v>179</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>180</v>
+      <c r="D27" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="E27" s="29" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="C28" s="36">
+        <v>174</v>
+      </c>
+      <c r="C28" s="35">
         <f>IFERROR(INC_cost_goods_sold/365,"")</f>
         <v>678053.44383561646</v>
       </c>
-      <c r="D28" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>183</v>
+      <c r="D28" s="29" t="s">
+        <v>175</v>
+      </c>
+      <c r="E28" s="29" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="35">
+        <v>60</v>
+      </c>
+      <c r="C29" s="34">
         <f>BAL_debt_long_term_curr</f>
         <v>224500548</v>
       </c>
-      <c r="D29" s="30" t="s">
-        <v>184</v>
-      </c>
-      <c r="E29" s="30" t="s">
-        <v>185</v>
+      <c r="D29" s="29" t="s">
+        <v>177</v>
+      </c>
+      <c r="E29" s="29" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="C30" s="35">
+        <v>179</v>
+      </c>
+      <c r="C30" s="34">
         <f>BAL_assets_current_curr-BAL_liabilities_current_curr</f>
         <v>71317900</v>
       </c>
-      <c r="D30" s="30" t="s">
-        <v>187</v>
-      </c>
-      <c r="E30" s="30" t="s">
-        <v>188</v>
+      <c r="D30" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="E30" s="29" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="C31" s="35">
+        <v>182</v>
+      </c>
+      <c r="C31" s="34">
         <f>BAL_assets_total_curr</f>
         <v>1118622625</v>
       </c>
-      <c r="D31" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="E31" s="30" t="s">
-        <v>191</v>
+      <c r="D31" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="E31" s="29" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="12" t="s">
-        <v>192</v>
-      </c>
-      <c r="C32" s="35">
+        <v>185</v>
+      </c>
+      <c r="C32" s="34">
         <f>BAL_debt_long_term_curr+BAL_equity_shareholders_curr</f>
         <v>375989483</v>
       </c>
-      <c r="D32" s="30" t="s">
-        <v>193</v>
-      </c>
-      <c r="E32" s="30" t="s">
-        <v>194</v>
+      <c r="D32" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="E32" s="29" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="12" t="s">
-        <v>195</v>
-      </c>
-      <c r="C33" s="35">
+        <v>188</v>
+      </c>
+      <c r="C33" s="34">
         <f>BAL_liabilities_total_curr</f>
         <v>967133690</v>
       </c>
-      <c r="D33" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="E33" s="30" t="s">
-        <v>197</v>
+      <c r="D33" s="29" t="s">
+        <v>189</v>
+      </c>
+      <c r="E33" s="29" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="53" t="s">
-        <v>198</v>
-      </c>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
+      <c r="B35" s="56" t="s">
+        <v>191</v>
+      </c>
+      <c r="C35" s="52"/>
+      <c r="D35" s="52"/>
+      <c r="E35" s="52"/>
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="C36" s="36">
+        <v>192</v>
+      </c>
+      <c r="C36" s="35">
         <f>AVERAGE(startYear_equity,currentYear_equity)</f>
         <v>152661708</v>
       </c>
-      <c r="D36" s="30" t="s">
-        <v>200</v>
-      </c>
-      <c r="E36" s="30" t="s">
-        <v>201</v>
+      <c r="D36" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="E36" s="29" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="C37" s="36">
+        <v>195</v>
+      </c>
+      <c r="C37" s="35">
         <f>AVERAGE(startYear_total_assets,currentYear_assets_total)</f>
         <v>977613264</v>
       </c>
-      <c r="D37" s="30" t="s">
-        <v>203</v>
-      </c>
-      <c r="E37" s="30" t="s">
-        <v>204</v>
+      <c r="D37" s="29" t="s">
+        <v>196</v>
+      </c>
+      <c r="E37" s="29" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="12" t="s">
-        <v>205</v>
-      </c>
-      <c r="C38" s="36">
+        <v>198</v>
+      </c>
+      <c r="C38" s="35">
         <f>AVERAGE(startYear_total_capitalization,currentYear_total_capitalization)</f>
         <v>331277438</v>
       </c>
-      <c r="D38" s="30" t="s">
-        <v>206</v>
-      </c>
-      <c r="E38" s="30" t="s">
-        <v>207</v>
+      <c r="D38" s="29" t="s">
+        <v>199</v>
+      </c>
+      <c r="E38" s="29" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="23" t="s">
-        <v>208</v>
-      </c>
-      <c r="C41" s="23" t="s">
-        <v>209</v>
-      </c>
-      <c r="D41" s="23" t="s">
-        <v>210</v>
-      </c>
-      <c r="E41" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="F41" s="23" t="s">
-        <v>211</v>
+      <c r="B41" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="C41" s="22" t="s">
+        <v>202</v>
+      </c>
+      <c r="D41" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="E41" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="F41" s="22" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="5" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -3498,37 +3478,37 @@
     </row>
     <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="C43" s="37"/>
-      <c r="D43" s="30" t="s">
-        <v>214</v>
-      </c>
-      <c r="E43" s="30"/>
+        <v>206</v>
+      </c>
+      <c r="C43" s="36"/>
+      <c r="D43" s="29" t="s">
+        <v>207</v>
+      </c>
+      <c r="E43" s="29"/>
     </row>
     <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="C44" s="38"/>
-      <c r="D44" s="30" t="s">
-        <v>216</v>
-      </c>
-      <c r="E44" s="30"/>
+        <v>208</v>
+      </c>
+      <c r="C44" s="37"/>
+      <c r="D44" s="29" t="s">
+        <v>209</v>
+      </c>
+      <c r="E44" s="29"/>
     </row>
     <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="12" t="s">
-        <v>217</v>
-      </c>
-      <c r="C45" s="37"/>
-      <c r="D45" s="30" t="s">
-        <v>218</v>
-      </c>
-      <c r="E45" s="30"/>
+        <v>210</v>
+      </c>
+      <c r="C45" s="36"/>
+      <c r="D45" s="29" t="s">
+        <v>211</v>
+      </c>
+      <c r="E45" s="29"/>
     </row>
     <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="5" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -3536,67 +3516,67 @@
     </row>
     <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="C47" s="39"/>
-      <c r="D47" s="30" t="s">
-        <v>221</v>
-      </c>
-      <c r="E47" s="30"/>
+        <v>213</v>
+      </c>
+      <c r="C47" s="38"/>
+      <c r="D47" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="E47" s="29"/>
     </row>
     <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="C48" s="39"/>
-      <c r="D48" s="30" t="s">
-        <v>223</v>
-      </c>
-      <c r="E48" s="30"/>
+        <v>215</v>
+      </c>
+      <c r="C48" s="38"/>
+      <c r="D48" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="E48" s="29"/>
     </row>
     <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="C49" s="39"/>
-      <c r="D49" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="E49" s="30"/>
+        <v>217</v>
+      </c>
+      <c r="C49" s="38"/>
+      <c r="D49" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="E49" s="29"/>
     </row>
     <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="C50" s="39"/>
-      <c r="D50" s="30" t="s">
-        <v>227</v>
-      </c>
-      <c r="E50" s="30"/>
+        <v>219</v>
+      </c>
+      <c r="C50" s="38"/>
+      <c r="D50" s="29" t="s">
+        <v>220</v>
+      </c>
+      <c r="E50" s="29"/>
     </row>
     <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="C51" s="39"/>
-      <c r="D51" s="30" t="s">
-        <v>229</v>
-      </c>
-      <c r="E51" s="30"/>
+        <v>221</v>
+      </c>
+      <c r="C51" s="38"/>
+      <c r="D51" s="29" t="s">
+        <v>222</v>
+      </c>
+      <c r="E51" s="29"/>
     </row>
     <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="C52" s="39"/>
-      <c r="D52" s="30" t="s">
-        <v>231</v>
-      </c>
-      <c r="E52" s="30"/>
+        <v>223</v>
+      </c>
+      <c r="C52" s="38"/>
+      <c r="D52" s="29" t="s">
+        <v>224</v>
+      </c>
+      <c r="E52" s="29"/>
     </row>
     <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -3604,81 +3584,81 @@
     </row>
     <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="12" t="s">
-        <v>233</v>
-      </c>
-      <c r="C54" s="38"/>
-      <c r="D54" s="30" t="s">
-        <v>234</v>
-      </c>
-      <c r="E54" s="30" t="s">
-        <v>235</v>
+        <v>226</v>
+      </c>
+      <c r="C54" s="37"/>
+      <c r="D54" s="29" t="s">
+        <v>227</v>
+      </c>
+      <c r="E54" s="29" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="12" t="s">
-        <v>236</v>
-      </c>
-      <c r="C55" s="38"/>
-      <c r="D55" s="30" t="s">
-        <v>237</v>
-      </c>
-      <c r="E55" s="30"/>
+        <v>229</v>
+      </c>
+      <c r="C55" s="37"/>
+      <c r="D55" s="29" t="s">
+        <v>230</v>
+      </c>
+      <c r="E55" s="29"/>
     </row>
     <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="C56" s="40"/>
-      <c r="D56" s="30" t="s">
-        <v>239</v>
-      </c>
-      <c r="E56" s="30"/>
+        <v>231</v>
+      </c>
+      <c r="C56" s="39"/>
+      <c r="D56" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="E56" s="29"/>
     </row>
     <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="C57" s="38"/>
-      <c r="D57" s="30" t="s">
-        <v>241</v>
-      </c>
-      <c r="E57" s="30"/>
+        <v>233</v>
+      </c>
+      <c r="C57" s="37"/>
+      <c r="D57" s="29" t="s">
+        <v>234</v>
+      </c>
+      <c r="E57" s="29"/>
     </row>
     <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="12" t="s">
-        <v>242</v>
-      </c>
-      <c r="C58" s="40"/>
-      <c r="D58" s="30" t="s">
-        <v>243</v>
-      </c>
-      <c r="E58" s="30"/>
+        <v>235</v>
+      </c>
+      <c r="C58" s="39"/>
+      <c r="D58" s="29" t="s">
+        <v>236</v>
+      </c>
+      <c r="E58" s="29"/>
     </row>
     <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="C59" s="39"/>
-      <c r="D59" s="30" t="s">
-        <v>245</v>
-      </c>
-      <c r="E59" s="30"/>
+        <v>237</v>
+      </c>
+      <c r="C59" s="38"/>
+      <c r="D59" s="29" t="s">
+        <v>238</v>
+      </c>
+      <c r="E59" s="29"/>
     </row>
     <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="C60" s="39"/>
-      <c r="D60" s="30" t="s">
-        <v>247</v>
-      </c>
-      <c r="E60" s="30" t="s">
-        <v>248</v>
+        <v>239</v>
+      </c>
+      <c r="C60" s="38"/>
+      <c r="D60" s="29" t="s">
+        <v>240</v>
+      </c>
+      <c r="E60" s="29" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="5" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -3686,81 +3666,81 @@
     </row>
     <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="12" t="s">
-        <v>250</v>
-      </c>
-      <c r="C62" s="39"/>
-      <c r="D62" s="30" t="s">
-        <v>251</v>
-      </c>
-      <c r="E62" s="30"/>
+        <v>243</v>
+      </c>
+      <c r="C62" s="38"/>
+      <c r="D62" s="29" t="s">
+        <v>244</v>
+      </c>
+      <c r="E62" s="29"/>
     </row>
     <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="12" t="s">
-        <v>252</v>
-      </c>
-      <c r="C63" s="38"/>
-      <c r="D63" s="30" t="s">
-        <v>253</v>
-      </c>
-      <c r="E63" s="30"/>
+        <v>245</v>
+      </c>
+      <c r="C63" s="37"/>
+      <c r="D63" s="29" t="s">
+        <v>246</v>
+      </c>
+      <c r="E63" s="29"/>
     </row>
     <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="C64" s="39"/>
-      <c r="D64" s="30" t="s">
-        <v>255</v>
-      </c>
-      <c r="E64" s="30"/>
+        <v>247</v>
+      </c>
+      <c r="C64" s="38"/>
+      <c r="D64" s="29" t="s">
+        <v>248</v>
+      </c>
+      <c r="E64" s="29"/>
     </row>
     <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="12" t="s">
-        <v>256</v>
-      </c>
-      <c r="C65" s="38"/>
-      <c r="D65" s="30" t="s">
-        <v>257</v>
-      </c>
-      <c r="E65" s="30"/>
+        <v>249</v>
+      </c>
+      <c r="C65" s="37"/>
+      <c r="D65" s="29" t="s">
+        <v>250</v>
+      </c>
+      <c r="E65" s="29"/>
     </row>
     <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="12" t="s">
-        <v>258</v>
-      </c>
-      <c r="C66" s="38"/>
-      <c r="D66" s="30" t="s">
-        <v>259</v>
-      </c>
-      <c r="E66" s="30"/>
+        <v>251</v>
+      </c>
+      <c r="C66" s="37"/>
+      <c r="D66" s="29" t="s">
+        <v>252</v>
+      </c>
+      <c r="E66" s="29"/>
     </row>
     <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="C67" s="41"/>
-      <c r="D67" s="30" t="s">
-        <v>261</v>
-      </c>
-      <c r="E67" s="30" t="s">
-        <v>262</v>
+        <v>253</v>
+      </c>
+      <c r="C67" s="40"/>
+      <c r="D67" s="29" t="s">
+        <v>254</v>
+      </c>
+      <c r="E67" s="29" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="12" t="s">
-        <v>263</v>
-      </c>
-      <c r="C68" s="38"/>
-      <c r="D68" s="30" t="s">
-        <v>264</v>
-      </c>
-      <c r="E68" s="30" t="s">
-        <v>265</v>
+        <v>256</v>
+      </c>
+      <c r="C68" s="37"/>
+      <c r="D68" s="29" t="s">
+        <v>257</v>
+      </c>
+      <c r="E68" s="29" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="5" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -3768,47 +3748,47 @@
     </row>
     <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="12" t="s">
-        <v>267</v>
-      </c>
-      <c r="C70" s="39"/>
-      <c r="D70" s="30" t="s">
-        <v>268</v>
-      </c>
-      <c r="E70" s="30"/>
+        <v>260</v>
+      </c>
+      <c r="C70" s="38"/>
+      <c r="D70" s="29" t="s">
+        <v>261</v>
+      </c>
+      <c r="E70" s="29"/>
     </row>
     <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="C71" s="38"/>
-      <c r="D71" s="30" t="s">
-        <v>270</v>
-      </c>
-      <c r="E71" s="30"/>
+        <v>262</v>
+      </c>
+      <c r="C71" s="37"/>
+      <c r="D71" s="29" t="s">
+        <v>263</v>
+      </c>
+      <c r="E71" s="29"/>
     </row>
     <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="C72" s="38"/>
-      <c r="D72" s="30" t="s">
-        <v>272</v>
-      </c>
-      <c r="E72" s="30"/>
+        <v>264</v>
+      </c>
+      <c r="C72" s="37"/>
+      <c r="D72" s="29" t="s">
+        <v>265</v>
+      </c>
+      <c r="E72" s="29"/>
     </row>
     <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="C73" s="38"/>
-      <c r="D73" s="30" t="s">
-        <v>274</v>
-      </c>
-      <c r="E73" s="30"/>
+        <v>266</v>
+      </c>
+      <c r="C73" s="37"/>
+      <c r="D73" s="29" t="s">
+        <v>267</v>
+      </c>
+      <c r="E73" s="29"/>
     </row>
     <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="5" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -3816,27 +3796,27 @@
     </row>
     <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="12" t="s">
-        <v>276</v>
-      </c>
-      <c r="C75" s="39"/>
-      <c r="D75" s="30" t="s">
-        <v>277</v>
-      </c>
-      <c r="E75" s="30"/>
-      <c r="F75" s="43" t="str">
+        <v>269</v>
+      </c>
+      <c r="C75" s="38"/>
+      <c r="D75" s="29" t="s">
+        <v>270</v>
+      </c>
+      <c r="E75" s="29"/>
+      <c r="F75" s="41" t="str">
         <f>IF(OR(C75="",C47=""),"",IF(ROUND(C75,6)=ROUND(C47,6),"✓ matches direct ROA","✗ differs by "&amp;TEXT(ABS(C75-C47),"0.00%")))</f>
         <v/>
       </c>
     </row>
     <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="C76" s="39"/>
-      <c r="D76" s="30" t="s">
-        <v>279</v>
-      </c>
-      <c r="E76" s="30"/>
+        <v>271</v>
+      </c>
+      <c r="C76" s="38"/>
+      <c r="D76" s="29" t="s">
+        <v>272</v>
+      </c>
+      <c r="E76" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3854,162 +3834,163 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="70" customWidth="1"/>
+    <col min="2" max="2" width="28" style="47" customWidth="1"/>
+    <col min="3" max="3" width="70" style="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="14" t="s">
+    <row r="2" spans="2:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="58" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="59" t="s">
+        <v>274</v>
+      </c>
+      <c r="C4" s="60" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="59" t="s">
+        <v>276</v>
+      </c>
+      <c r="C5" s="60" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="59" t="s">
+        <v>278</v>
+      </c>
+      <c r="C6" s="61" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="59" t="s">
+        <v>279</v>
+      </c>
+      <c r="C7" s="61" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="59" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="42" t="s">
+      <c r="C8" s="61" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="59" t="s">
         <v>281</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C9" s="61" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="59" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="42" t="s">
+      <c r="C10" s="61" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="59" t="s">
         <v>283</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C11" s="61" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" ht="96.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="59" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="42" t="s">
+      <c r="C12" s="61" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="59" t="s">
         <v>285</v>
       </c>
-      <c r="C6" s="44" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="42" t="s">
+      <c r="C13" s="61" t="s">
         <v>286</v>
       </c>
-      <c r="C7" s="44" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="42" t="s">
+    </row>
+    <row r="14" spans="2:3" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="59" t="s">
         <v>287</v>
       </c>
-      <c r="C8" s="44" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="B9" s="42" t="s">
+      <c r="C14" s="61" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="59" t="s">
         <v>288</v>
       </c>
-      <c r="C9" s="44" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B10" s="42" t="s">
+      <c r="C15" s="60" t="s">
         <v>289</v>
       </c>
-      <c r="C10" s="44" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B11" s="42" t="s">
+    </row>
+    <row r="16" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="59" t="s">
         <v>290</v>
       </c>
-      <c r="C11" s="44" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" ht="90" x14ac:dyDescent="0.25">
-      <c r="B12" s="42" t="s">
+      <c r="C16" s="60" t="s">
         <v>291</v>
       </c>
-      <c r="C12" s="44" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="13" spans="2:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B13" s="42" t="s">
+    </row>
+    <row r="17" spans="2:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="B17" s="59" t="s">
         <v>292</v>
       </c>
-      <c r="C13" s="44" t="s">
+      <c r="C17" s="60" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="B14" s="42" t="s">
+    <row r="18" spans="2:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="59" t="s">
         <v>294</v>
       </c>
-      <c r="C14" s="44" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="42" t="s">
+      <c r="C18" s="60" t="s">
         <v>295</v>
       </c>
-      <c r="C15" s="4" t="s">
+    </row>
+    <row r="19" spans="2:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="59" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="16" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="42" t="s">
+      <c r="C19" s="60" t="s">
         <v>297</v>
       </c>
-      <c r="C16" s="4" t="s">
+    </row>
+    <row r="20" spans="2:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="59" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="17" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="42" t="s">
+      <c r="C20" s="62"/>
+    </row>
+    <row r="21" spans="2:3" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="59" t="s">
         <v>299</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C21" s="60" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="42" t="s">
+    <row r="22" spans="2:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="B22" s="59" t="s">
         <v>301</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C22" s="60" t="s">
         <v>302</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="42" t="s">
-        <v>303</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="42" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="42" t="s">
-        <v>306</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="42" t="s">
-        <v>308</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>